<commit_message>
v0.22: unify CDSS as SST, clarify MBI in MRE label
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXuBp5SMoG4pD1jWH8rtoe
</commit_message>
<xml_diff>
--- a/output/central_unit_requests/MRE - SR26 sustainability reporting request.xlsx
+++ b/output/central_unit_requests/MRE - SR26 sustainability reporting request.xlsx
@@ -664,7 +664,7 @@
 • Where a related end-2025 target existed, click the ref in Column H to see your full SR25 response (Tab 3)
 • Use Tab 2 of this spreadsheet to highlight key sustainability stories (optional)
 • 2026 is a transition year: Sustainability 2030 launched ~20 October 2026, so report on activity across all of 2026 and any early actions since launch. No target status rating is requested this year.
-• Due: Tuesday 15 December 2026. Questions: CDSS – questions and clarifications are recorded centrally (contact email TBC); optional 1:1 meetings available on request</t>
+• Due: Tuesday 15 December 2026. Questions: Sustainability Strategy team (SST) – questions and clarifications are recorded centrally (contact email TBC); optional 1:1 meetings available on request</t>
         </is>
       </c>
     </row>
@@ -677,7 +677,7 @@
     <row r="11" ht="39" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>MRE – Research (incl. MBI – TBC)</t>
+          <t>MRE – Research (incl. MBI for NB2(a) nature footprint)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v0.27: MRE one row per research indicator; MBI/NB2(a) removed from MRE
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXuBp5SMoG4pD1jWH8rtoe
</commit_message>
<xml_diff>
--- a/output/central_unit_requests/MRE - SR26 sustainability reporting request.xlsx
+++ b/output/central_unit_requests/MRE - SR26 sustainability reporting request.xlsx
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.##"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -107,6 +107,13 @@
       <sz val="10"/>
     </font>
     <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
       <name val="Aptos"/>
       <b val="1"/>
     </font>
@@ -181,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -218,11 +225,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -737,7 +747,7 @@
     <outlinePr summaryBelow="1" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -833,7 +843,7 @@
     <row r="11" ht="39" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>MRE – Melbourne Research and Enterprise (incl. Melbourne Biodiversity Institute for NB2(a))</t>
+          <t>MRE – Melbourne Research and Enterprise</t>
         </is>
       </c>
     </row>
@@ -959,10 +969,10 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="409" customHeight="1">
+    <row r="16" ht="188" customHeight="1">
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>TR1(a)–(d)</t>
+          <t>TR1(a)</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
@@ -977,47 +987,47 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>(a) Expert-reviewed evidence of researchers contributing to operational sustainability priorities through partnerships, advisory input, living labs, applied projects or decision-support
-(b) Evidence of institutional pathways that enable ongoing collaboration between academic and professional staff
-(c) Expert assessment of the quality, relevance and continuity of these collaborations
-(d) Periodic feedback from participants on the effectiveness and mutual benefit of collaboration mechanisms.</t>
+          <t>Expert-reviewed evidence of researchers contributing to operational sustainability priorities through partnerships, advisory input, living labs, applied projects or decision-support</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>Melbourne Research and Enterprise (MRE) prepared the research targets, so we are asking about every indicator under this target, University-wide. Please respond to each part (a)–(d):
-(a) Expert-reviewed evidence of researchers contributing to operational sustainability priorities through partnerships, advisory input, living labs, applied projects or decision-support
-→ Please provide examples of researchers across the University contributing to University operational sustainability priorities through partnerships, advisory input, living labs, applied projects or decision-support. Briefly describe the operational challenge, researcher contribution and resulting or expected outcome.
-(b) Evidence of institutional pathways that enable ongoing collaboration between academic and professional staff
-→ Please describe any pathways, mechanisms or processes across the University that enable ongoing collaboration between academic and professional staff on operational sustainability challenges, could include formal programs, governance arrangements, funding mechanisms or coordination channels.
-(c) Expert assessment of the quality, relevance and continuity of these collaborations
-→ Please provide an assessment of the quality, relevance and continuity of sustainability-related collaborations involving the University, could include evidence of whether collaborations are sustained, useful to operational priorities and producing relevant outcomes.
-(d) Periodic feedback from participants on the effectiveness and mutual benefit of collaboration mechanisms.
-→ Please provide any participant feedback or other evidence from across the University on the effectiveness and mutual benefit of collaboration mechanisms between researchers and operational teams, could include key findings and any improvements identified.</t>
+          <t>Please provide examples of researchers across the University contributing to University operational sustainability priorities through partnerships, advisory input, living labs, applied projects or decision-support. Briefly describe the operational challenge, researcher contribution and resulting or expected outcome.
+In end-2025 reporting your area reported on the related SP2030 target 5a(i) (click the ref in Column H to see it in full in Tab 3).</t>
         </is>
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>We will report on examples of researchers helping solve the University's own operational sustainability challenges, alongside Campus Living Lab Accelerator Program case studies collected directly from project owners, and share them with operational teams to identify further collaboration. We will map existing academic–professional collaboration mechanisms across faculties to establish a baseline for this new indicator and identify models other faculties could adopt. We will use your assessment to describe the quality and continuity of research–operations collaboration in the 2026 report, and as baseline evidence for the interim target status assessment from 2027. We will use any feedback to understand whether collaboration mechanisms are working and to inform improvements. Where none has been collected, this helps us plan how to gather feedback from 2027.</t>
-        </is>
-      </c>
-      <c r="H16" s="13" t="inlineStr">
-        <is>
-          <t>N/A – new indicator</t>
-        </is>
-      </c>
-      <c r="I16" s="13" t="inlineStr"/>
-      <c r="J16" s="13" t="inlineStr"/>
+          <t>We will report on examples of researchers helping solve the University's own operational sustainability challenges, alongside Campus Living Lab Accelerator Program case studies collected directly from project owners, and share them with operational teams to identify further collaboration.</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t>5a(i)
+→ view SR25 response</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>"The Melbourne Biodiversity Institute launched, with academic and professional staff at the University collaborating to enhance biodiversity outcomes on and beyond our campuses. In its first year MBI secured funds alongside local and national partners, and advanced 12 biodiversity projects with real-world outcomes. With partners spanning government, business and finance, energy and sustainability, organisations, research outcomes from the institute inlude assessing whether carbon and biodiversisty markets support First Peoples caring for Country, rapid energy transitions and renewables infrastructure. 
+We are implementing our new Research Strategy 'Advancing Research 2030 - Excellence for Impact' with a key initiative 'Melbourne Impact Accelerators' designed to address the complex challenges we face and deliver lasting impact. A key Impact Accelerator is 'Climate Sustainability and Ecosystem Health'.  The research will help build resilience, support new energy transitions, improve biodiversity, help reverse habitat loss and contribute to effective policy. " Implementation is underway over 2026 and 2027.</t>
+        </is>
+      </c>
       <c r="K16" s="13" t="inlineStr"/>
-      <c r="L16" s="14" t="n"/>
-      <c r="M16" s="14" t="n"/>
-      <c r="N16" s="14" t="n"/>
-      <c r="O16" s="14" t="n"/>
-    </row>
-    <row r="17" ht="409" customHeight="1">
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="15" t="n"/>
+      <c r="N16" s="15" t="n"/>
+      <c r="O16" s="15" t="n"/>
+    </row>
+    <row r="17" ht="150" customHeight="1">
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>TR2(a)–(d)</t>
+          <t>TR1(b)</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
@@ -1027,33 +1037,22 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Deliver high-quality research and partnerships that contribute to sustainability outcomes and demonstrable societal benefit.</t>
+          <t>Utilise the expertise of the University’s researchers through mutually beneficial partnerships to help address the University’s operational sustainability challenges.</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>(a) Evidence of sustainability-related research impact across diverse pathways, could include policy, industry, community, practice, cultural and institutional outcomes
-(b) Documented progress of relevant strategic initiatives, including Impact Accelerators
-(c) Expert-reviewed summary of sustainability-related research outputs, outcomes and influence using available institutional evidence sources
-(d) Case-based evidence demonstrating how research has contributed to meaningful sustainability outcomes.</t>
+          <t>Evidence of institutional pathways that enable ongoing collaboration between academic and professional staff</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Please respond to each part (a)–(d), University-wide:
-(a) Evidence of sustainability-related research impact across diverse pathways, could include policy, industry, community, practice, cultural and institutional outcomes
-→ Please provide examples of sustainability-related research impact from across the University in policy, industry, community, practice, cultural or institutional pathways. For key examples, briefly describe the research contribution, partner/user and resulting outcome or influence.
-(b) Documented progress of relevant strategic initiatives, including Impact Accelerators
-→ Please provide case studies demonstrating how University research has contributed to meaningful sustainability outcomes. For each case, briefly describe the research, stakeholders involved, pathway to impact and evidence of the resulting sustainability outcome.
-(c) Expert-reviewed summary of sustainability-related research outputs, outcomes and influence using available institutional evidence sources
-→ Please prepare the SciVal and Altmetric output on sustainability-related research (e.g. SDG-mapped publications), as previously prepared by Shane Wood. Quantitative figures are requested in Tab 4 (Quantitative data).
-(d) Case-based evidence demonstrating how research has contributed to meaningful sustainability outcomes.
-→ Please provide case studies from across the University demonstrating how research has contributed to meaningful sustainability outcomes. Briefly describe the research, stakeholders involved, pathway to impact and evidence of the resulting sustainability outcome.</t>
+          <t>Please describe any pathways, mechanisms or processes across the University that enable ongoing collaboration between academic and professional staff on operational sustainability challenges, could include formal programs, governance arrangements, funding mechanisms or coordination channels.</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>We will collate research impact examples across faculties to show the breadth of sustainability-related research impact in the Transformational research section of the 2026 Sustainability Report, complementing University-wide metrics from Melbourne Research and Enterprise (MRE). We will use this to inform the Transformational research section of the 2026 Sustainability Report (transition year), and to establish a baseline for reporting against Sustainability 2030 from 2027. Strong examples may be followed up as case studies. We will use institutional research output data (e.g. SDG-mapped publications via SciVal) to provide the University-wide quantitative picture of sustainability-related research in the 2026 Sustainability Report. We will select the strongest examples to develop as full research case studies for the 2026 Sustainability Report (we may contact you for more detail and imag</t>
+          <t>We will map existing academic–professional collaboration mechanisms across faculties to establish a baseline for this new indicator and identify models other faculties could adopt.</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
@@ -1064,15 +1063,15 @@
       <c r="I17" s="13" t="inlineStr"/>
       <c r="J17" s="13" t="inlineStr"/>
       <c r="K17" s="13" t="inlineStr"/>
-      <c r="L17" s="14" t="n"/>
-      <c r="M17" s="14" t="n"/>
-      <c r="N17" s="14" t="n"/>
-      <c r="O17" s="14" t="n"/>
-    </row>
-    <row r="18" ht="409" customHeight="1">
+      <c r="L17" s="15" t="n"/>
+      <c r="M17" s="15" t="n"/>
+      <c r="N17" s="15" t="n"/>
+      <c r="O17" s="15" t="n"/>
+    </row>
+    <row r="18" ht="150" customHeight="1">
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>TR3(a)–(d)</t>
+          <t>TR1(c)</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
@@ -1082,33 +1081,22 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Embed sustainability within research systems, processes, capability and culture, so research is conducted responsibly, efficiently and with reduced environmental impact.</t>
+          <t>Utilise the expertise of the University’s researchers through mutually beneficial partnerships to help address the University’s operational sustainability challenges.</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>(a) Evidence that sustainability considerations are integrated into relevant research systems, planning processes, guidance, training, induction or support services
-(b) Demonstrated examples of more sustainable research practices in laboratories, fieldwork, procurement, travel or infrastructure use
-(c) Evidence of progress in sustainability-related research culture, capability and awareness, informed by periodic staff and graduate researcher surveys
-(d) Expert assessment of progress in embedding sustainable research practices across the institution.</t>
+          <t>Expert assessment of the quality, relevance and continuity of these collaborations</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>MRE is responsible for this target at a University-wide level. For each part (a)–(d), please describe progress within MRE and progress across the University:
-(a) Evidence that sustainability considerations are integrated into relevant research systems, planning processes, guidance, training, induction or support services
-→ Please describe how sustainability considerations are integrated into research systems, planning processes, guidance, training, induction or support services within MRE and across the University, could include examples of any new or improved processes.
-(b) Demonstrated examples of more sustainable research practices in laboratories, fieldwork, procurement, travel or infrastructure use
-→ Please describe any efforts within MRE and across the University to make research practices more sustainable, could include examples from laboratories, fieldwork, procurement, research travel or infrastructure use. Where available, provide evidence of uptake, resource savings, emissions reductions or other outcomes.
-(c) Evidence of progress in sustainability-related research culture, capability and awareness, informed by periodic staff and graduate researcher surveys
-→ Please provide evidence of progress in sustainability-related research culture, capability and awareness within MRE and across the University. This could include relevant staff and/or graduate researcher survey findings, participation in capability-building activities, or other indicators of change over time.
-(d) Expert assessment of progress in embedding sustainable research practices across the institution.
-→ An assessment of progress in embedding sustainable research practices, highlighting areas of strong progress, remaining gaps and priority actions for further improvement.</t>
+          <t>Please provide an assessment of the quality, relevance and continuity of sustainability-related collaborations involving the University, could include evidence of whether collaborations are sustained, useful to operational priorities and producing relevant outcomes.</t>
         </is>
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>We will report on how sustainability is being built into research systems and support across the University, and use responses to establish a baseline for this new target. We will report on ways the University is making research practices more sustainable in the 2026 Sustainability Report, and share practical examples (e.g. green labs) across faculties. We will use any survey or capability data to describe changes in sustainability-related research culture. Where no evidence exists, this helps us plan University-wide measurement (e.g. staff and graduate researcher surveys) from 2027. We will use faculty self-assessments to identify strengths, gaps and priority actions in embedding sustainable research practices, to inform internal management reporting and the Transformational research working group.</t>
+          <t>We will use your assessment to describe the quality and continuity of research–operations collaboration in the 2026 report, and as baseline evidence for the interim target status assessment from 2027.</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
@@ -1119,41 +1107,40 @@
       <c r="I18" s="13" t="inlineStr"/>
       <c r="J18" s="13" t="inlineStr"/>
       <c r="K18" s="13" t="inlineStr"/>
-      <c r="L18" s="14" t="n"/>
-      <c r="M18" s="14" t="n"/>
-      <c r="N18" s="14" t="n"/>
-      <c r="O18" s="14" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
+      <c r="N18" s="15" t="n"/>
+      <c r="O18" s="15" t="n"/>
     </row>
     <row r="19" ht="150" customHeight="1">
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>NB2(a)</t>
+          <t>TR1(d)</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Nature and biodiversity</t>
+          <t>Transformational research</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Improve our understanding of our supply chain impacts on nature.</t>
+          <t>Utilise the expertise of the University’s researchers through mutually beneficial partnerships to help address the University’s operational sustainability challenges.</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Documented baseline nature footprint analysis</t>
+          <t>Periodic feedback from participants on the effectiveness and mutual benefit of collaboration mechanisms.</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>Impact Encore Measurement
-Quantitative figures for this indicator are requested separately in Tab 4 (Quantitative data).</t>
+          <t>Please provide any participant feedback or other evidence from across the University on the effectiveness and mutual benefit of collaboration mechanisms between researchers and operational teams, could include key findings and any improvements identified.</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>We will report on the baseline nature footprint of the University's supply chain in the Nature and biodiversity section of the 2026 Sustainability Report.</t>
+          <t>We will use any feedback to understand whether collaboration mechanisms are working and to inform improvements. Where none has been collected, this helps us plan how to gather feedback from 2027.</t>
         </is>
       </c>
       <c r="H19" s="13" t="inlineStr">
@@ -1164,12 +1151,411 @@
       <c r="I19" s="13" t="inlineStr"/>
       <c r="J19" s="13" t="inlineStr"/>
       <c r="K19" s="13" t="inlineStr"/>
-      <c r="L19" s="14" t="n"/>
-      <c r="M19" s="14" t="n"/>
-      <c r="N19" s="14" t="n"/>
-      <c r="O19" s="14" t="n"/>
-    </row>
-    <row r="20"/>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="15" t="n"/>
+      <c r="N19" s="15" t="n"/>
+      <c r="O19" s="15" t="n"/>
+    </row>
+    <row r="20" ht="171" customHeight="1">
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>TR2(a)</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Transformational research</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Deliver high-quality research and partnerships that contribute to sustainability outcomes and demonstrable societal benefit.</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Evidence of sustainability-related research impact across diverse pathways, could include policy, industry, community, practice, cultural and institutional outcomes</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>Please provide examples of sustainability-related research impact from across the University in policy, industry, community, practice, cultural or institutional pathways. For key examples, briefly describe the research contribution, partner/user and resulting outcome or influence.
+In end-2025 reporting your area reported on the related SP2030 target 5b(ii) (click the ref in Column H to see it in full in Tab 3).</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>We will collate research impact examples across faculties to show the breadth of sustainability-related research impact in the Transformational research section of the 2026 Sustainability Report, complementing University-wide metrics from Melbourne Research and Enterprise (MRE).</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t>5b(ii)
+→ view SR25 response</t>
+        </is>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>The University’s research outputs continue to be extensively mentioned in patents, policy, news and social media. Data is below on University research outputs for 2025 so far.</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr"/>
+      <c r="L20" s="15" t="n"/>
+      <c r="M20" s="15" t="n"/>
+      <c r="N20" s="15" t="n"/>
+      <c r="O20" s="15" t="n"/>
+    </row>
+    <row r="21" ht="150" customHeight="1">
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>TR2(b)</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Transformational research</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Deliver high-quality research and partnerships that contribute to sustainability outcomes and demonstrable societal benefit.</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>Documented progress of relevant strategic initiatives, including Impact Accelerators</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Please provide case studies demonstrating how University research has contributed to meaningful sustainability outcomes. For each case, briefly describe the research, stakeholders involved, pathway to impact and evidence of the resulting sustainability outcome.
+Quantitative figures for this indicator are requested separately in Tab 4 (Quantitative data).</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>We will use this to inform the Transformational research section of the 2026 Sustainability Report (transition year), and to establish a baseline for reporting against Sustainability 2030 from 2027. Strong examples may be followed up as case studies.</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>N/A – new indicator</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="inlineStr"/>
+      <c r="J21" s="13" t="inlineStr"/>
+      <c r="K21" s="13" t="inlineStr"/>
+      <c r="L21" s="15" t="n"/>
+      <c r="M21" s="15" t="n"/>
+      <c r="N21" s="15" t="n"/>
+      <c r="O21" s="15" t="n"/>
+    </row>
+    <row r="22" ht="171" customHeight="1">
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>TR2(c)</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Transformational research</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Deliver high-quality research and partnerships that contribute to sustainability outcomes and demonstrable societal benefit.</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>Expert-reviewed summary of sustainability-related research outputs, outcomes and influence using available institutional evidence sources</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Please prepare the SciVal and Altmetric output on sustainability-related research (e.g. SDG-mapped publications), as previously prepared by Shane Wood.
+In end-2025 reporting your area reported on the related SP2030 target 5b(iii) (click the ref in Column H to see it in full in Tab 3).
+Quantitative figures for this indicator are requested separately in Tab 4 (Quantitative data).</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="inlineStr">
+        <is>
+          <t>We will use institutional research output data (e.g. SDG-mapped publications via SciVal) to provide the University-wide quantitative picture of sustainability-related research in the 2026 Sustainability Report.</t>
+        </is>
+      </c>
+      <c r="H22" s="14" t="inlineStr">
+        <is>
+          <t>5b(iii)
+→ view SR25 response</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>The University’s research outputs continue to be extensively mentioned in patents, policy, news and social media.</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="inlineStr"/>
+      <c r="L22" s="15" t="n"/>
+      <c r="M22" s="15" t="n"/>
+      <c r="N22" s="15" t="n"/>
+      <c r="O22" s="15" t="n"/>
+    </row>
+    <row r="23" ht="150" customHeight="1">
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>TR2(d)</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Transformational research</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Deliver high-quality research and partnerships that contribute to sustainability outcomes and demonstrable societal benefit.</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>Case-based evidence demonstrating how research has contributed to meaningful sustainability outcomes.</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Please provide case studies from across the University demonstrating how research has contributed to meaningful sustainability outcomes. Briefly describe the research, stakeholders involved, pathway to impact and evidence of the resulting sustainability outcome.</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>We will select the strongest examples to develop as full research case studies for the 2026 Sustainability Report (we may contact you for more detail and images).</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>N/A – new indicator</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="inlineStr"/>
+      <c r="J23" s="13" t="inlineStr"/>
+      <c r="K23" s="13" t="inlineStr"/>
+      <c r="L23" s="15" t="n"/>
+      <c r="M23" s="15" t="n"/>
+      <c r="N23" s="15" t="n"/>
+      <c r="O23" s="15" t="n"/>
+    </row>
+    <row r="24" ht="220" customHeight="1">
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>TR3(a)</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Transformational research</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Embed sustainability within research systems, processes, capability and culture, so research is conducted responsibly, efficiently and with reduced environmental impact.</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>Evidence that sustainability considerations are integrated into relevant research systems, planning processes, guidance, training, induction or support services</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>MRE is responsible for this target at a University-wide level – please describe progress within MRE and progress across the University.
+Please describe how sustainability considerations are integrated into research systems, planning processes, guidance, training, induction or support services across the University, could include examples of any new or improved processes.
+In end-2025 reporting your area reported on the related SP2030 target 5c(i) (click the ref in Column H to see it in full in Tab 3).</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="inlineStr">
+        <is>
+          <t>We will report on how sustainability is being built into research systems and support across the University, and use responses to establish a baseline for this new target.</t>
+        </is>
+      </c>
+      <c r="H24" s="14" t="inlineStr">
+        <is>
+          <t>5c(i)
+→ view SR25 response</t>
+        </is>
+      </c>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>We continue to encourage all researchers at the University to consider the impacts of their research, including in relation to sustainability through the Research in a Publicly Spirited University, and Openness Transparency agenda in the new Research Strategy.</t>
+        </is>
+      </c>
+      <c r="K24" s="13" t="inlineStr"/>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="15" t="n"/>
+      <c r="N24" s="15" t="n"/>
+      <c r="O24" s="15" t="n"/>
+    </row>
+    <row r="25" ht="286" customHeight="1">
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>TR3(b)</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Transformational research</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Embed sustainability within research systems, processes, capability and culture, so research is conducted responsibly, efficiently and with reduced environmental impact.</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>Demonstrated examples of more sustainable research practices in laboratories, fieldwork, procurement, travel or infrastructure use</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>MRE is responsible for this target at a University-wide level – please describe progress within MRE and progress across the University.
+Please describe any efforts across the University to make research practices more sustainable, could include examples from laboratories, fieldwork, procurement, research travel or infrastructure use. Where available, provide evidence of uptake, resource savings, emissions reductions or other outcomes.
+In end-2025 reporting your area reported on the related SP2030 target 5c(ii) (click the ref in Column H to see it in full in Tab 3).
+Quantitative figures for this indicator are requested separately in Tab 4 (Quantitative data).</t>
+        </is>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>We will report on ways the University is making research practices more sustainable in the 2026 Sustainability Report, and share practical examples (e.g. green labs) across faculties.</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>5c(ii)
+→ view SR25 response</t>
+        </is>
+      </c>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr">
+        <is>
+          <t>We continue to hold seminars, with professionals and academics to discuss opportunities to expand our sustainability efforts across the University. Initiatives like the MCF Seminar Series, a series of seminars designed to bring together researchers, practitioners, and the public to discuss various aspects of climate change and sustainability, continues its third year as Melbourne Connect, with Academics and Professionals alike in attendance. Deep-Dive sessions are also held with colleagues to discuss sustainability impacts and initiatives, presented by the Sustainability Team.</t>
+        </is>
+      </c>
+      <c r="K25" s="13" t="inlineStr"/>
+      <c r="L25" s="15" t="n"/>
+      <c r="M25" s="15" t="n"/>
+      <c r="N25" s="15" t="n"/>
+      <c r="O25" s="15" t="n"/>
+    </row>
+    <row r="26" ht="171" customHeight="1">
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>TR3(c)</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Transformational research</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Embed sustainability within research systems, processes, capability and culture, so research is conducted responsibly, efficiently and with reduced environmental impact.</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>Evidence of progress in sustainability-related research culture, capability and awareness, informed by periodic staff and graduate researcher surveys</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>MRE is responsible for this target at a University-wide level – please describe progress within MRE and progress across the University.
+Please provide evidence of progress in sustainability-related research culture, capability and awareness across the University. This could include relevant staff and/or graduate researcher survey findings, participation in capability-building activities, or other indicators of change over time.</t>
+        </is>
+      </c>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>We will use any survey or capability data to describe changes in sustainability-related research culture. Where no evidence exists, this helps us plan University-wide measurement (e.g. staff and graduate researcher surveys) from 2027.</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="inlineStr">
+        <is>
+          <t>N/A – new indicator</t>
+        </is>
+      </c>
+      <c r="I26" s="13" t="inlineStr"/>
+      <c r="J26" s="13" t="inlineStr"/>
+      <c r="K26" s="13" t="inlineStr"/>
+      <c r="L26" s="15" t="n"/>
+      <c r="M26" s="15" t="n"/>
+      <c r="N26" s="15" t="n"/>
+      <c r="O26" s="15" t="n"/>
+    </row>
+    <row r="27" ht="150" customHeight="1">
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>TR3(d)</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Transformational research</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Embed sustainability within research systems, processes, capability and culture, so research is conducted responsibly, efficiently and with reduced environmental impact.</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>Expert assessment of progress in embedding sustainable research practices across the institution.</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>MRE is responsible for this target at a University-wide level – please describe progress within MRE and progress across the University.
+An assessment of progress in embedding sustainable research practices, highlighting areas of strong progress, remaining gaps and priority actions for further improvement.</t>
+        </is>
+      </c>
+      <c r="G27" s="13" t="inlineStr">
+        <is>
+          <t>We will use faculty self-assessments to identify strengths, gaps and priority actions in embedding sustainable research practices, to inform internal management reporting and the Transformational research working group.</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="inlineStr">
+        <is>
+          <t>N/A – new indicator</t>
+        </is>
+      </c>
+      <c r="I27" s="13" t="inlineStr"/>
+      <c r="J27" s="13" t="inlineStr"/>
+      <c r="K27" s="13" t="inlineStr"/>
+      <c r="L27" s="15" t="n"/>
+      <c r="M27" s="15" t="n"/>
+      <c r="N27" s="15" t="n"/>
+      <c r="O27" s="15" t="n"/>
+    </row>
+    <row r="28"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="4">
@@ -1178,6 +1564,13 @@
     <mergeCell ref="D4:G8"/>
     <mergeCell ref="B4:C8"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H16" location="'3. SR25 responses'!B8"/>
+    <hyperlink ref="H20" location="'3. SR25 responses'!B11"/>
+    <hyperlink ref="H22" location="'3. SR25 responses'!B10"/>
+    <hyperlink ref="H24" location="'3. SR25 responses'!B13"/>
+    <hyperlink ref="H25" location="'3. SR25 responses'!B14"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -1259,12 +1652,12 @@
     <row r="3"/>
     <row r="4"/>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>How to use this spreadsheet</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>Please share up to 3 stories from 2026 which highlight your faculty's/portfolio's sustainability progress and/or impact. These stories can directly relate to Sustainability 2030 targets and indicators, or sustainability more generally. Due: Thursday 24 December 2026 (Christmas shutdown) (early submission helps us develop case studies).</t>
         </is>
@@ -1273,77 +1666,77 @@
     <row r="6"/>
     <row r="7"/>
     <row r="8" ht="39" customHeight="1">
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Related Sustainability 2030 targets (optional)</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>Images and other media</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr">
+      <c r="F8" s="18" t="inlineStr">
         <is>
           <t>Links and supporting documentation</t>
         </is>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1">
-      <c r="B9" s="18" t="inlineStr"/>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr"/>
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>• Please include a brief description of a project or activity that has made a significant contribution to sustainability at the University (up to 250 words)
 • Summarise the benefits. Benefits may relate to operational outcomes, environmental/social outcomes, and sector benefits.</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr"/>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr"/>
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>(link to OneDrive/SharePoint files or published online content preferred)</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr"/>
+      <c r="F9" s="19" t="inlineStr"/>
     </row>
     <row r="10" ht="120" customHeight="1">
       <c r="A10" t="n">
         <v>1</v>
       </c>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="14" t="n"/>
-      <c r="E10" s="14" t="n"/>
-      <c r="F10" s="14" t="n"/>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
     </row>
     <row r="11" ht="120" customHeight="1">
       <c r="A11" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="14" t="n"/>
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="14" t="n"/>
-      <c r="F12" s="14" t="n"/>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
@@ -1429,21 +1822,21 @@
       <c r="R2" s="1" t="n"/>
     </row>
     <row r="3" ht="32" customHeight="1">
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>Your responses to the end-2025 reporting request, against the former Sustainability Plan 2030 (SP2030) targets. For reference only – please do not edit. Use the 'Back to request' links to return to the reporting template.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>← Back to request</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Chancellery Research and Enterprise</t>
         </is>
@@ -1775,7 +2168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R111"/>
+  <dimension ref="A1:R104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1843,7 +2236,7 @@
       <c r="R2" s="1" t="n"/>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>These figures feed the Sustainability Databook (the University's authoritative quantitative source). Previous years are shown for context – please do not alter. Please provide the CY2026 value (provisional or year-to-date figures are fine; we will confirm final figures with you in January–February), the data source, and any change to definition or boundary. Due: Thursday 24 December 2026 (Christmas shutdown).</t>
         </is>
@@ -1935,72 +2328,72 @@
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>No instructions – context only.</t>
         </is>
       </c>
-      <c r="C7" s="21" t="inlineStr"/>
-      <c r="D7" s="21" t="inlineStr"/>
-      <c r="E7" s="21" t="inlineStr"/>
-      <c r="F7" s="21" t="inlineStr"/>
-      <c r="G7" s="21" t="inlineStr"/>
-      <c r="H7" s="21" t="inlineStr"/>
-      <c r="I7" s="21" t="inlineStr"/>
-      <c r="J7" s="21" t="inlineStr"/>
-      <c r="K7" s="21" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr"/>
+      <c r="D7" s="22" t="inlineStr"/>
+      <c r="E7" s="22" t="inlineStr"/>
+      <c r="F7" s="22" t="inlineStr"/>
+      <c r="G7" s="22" t="inlineStr"/>
+      <c r="H7" s="22" t="inlineStr"/>
+      <c r="I7" s="22" t="inlineStr"/>
+      <c r="J7" s="22" t="inlineStr"/>
+      <c r="K7" s="22" t="inlineStr">
         <is>
           <t>Please enter numerical values</t>
         </is>
       </c>
-      <c r="L7" s="21" t="inlineStr">
+      <c r="L7" s="22" t="inlineStr">
         <is>
           <t>Please provide a file name or link to the data source</t>
         </is>
       </c>
-      <c r="M7" s="21" t="inlineStr">
+      <c r="M7" s="22" t="inlineStr">
         <is>
           <t>Describe any change since last year (or 'No change')</t>
         </is>
       </c>
-      <c r="N7" s="21" t="inlineStr">
+      <c r="N7" s="22" t="inlineStr">
         <is>
           <t>Please add any additional notes here</t>
         </is>
       </c>
-      <c r="O7" s="21" t="inlineStr">
+      <c r="O7" s="22" t="inlineStr">
         <is>
           <t>Please provide information on any useful case studies</t>
         </is>
       </c>
     </row>
     <row r="8" ht="56" customHeight="1">
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>TR2(b)</t>
         </is>
       </c>
-      <c r="C8" s="22" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>Documented progress of relevant strategic initiatives, including Impact Accelerators</t>
         </is>
       </c>
-      <c r="D8" s="22" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>Completion rate to the set annual target of strategic initiatives</t>
         </is>
       </c>
-      <c r="E8" s="22" t="inlineStr"/>
-      <c r="F8" s="23" t="n"/>
-      <c r="G8" s="23" t="n"/>
-      <c r="H8" s="23" t="n"/>
-      <c r="I8" s="23" t="n"/>
-      <c r="J8" s="22" t="inlineStr"/>
-      <c r="K8" s="24" t="n"/>
-      <c r="L8" s="24" t="n"/>
-      <c r="M8" s="24" t="n"/>
-      <c r="N8" s="24" t="n"/>
-      <c r="O8" s="24" t="n"/>
+      <c r="E8" s="23" t="inlineStr"/>
+      <c r="F8" s="24" t="n"/>
+      <c r="G8" s="24" t="n"/>
+      <c r="H8" s="24" t="n"/>
+      <c r="I8" s="24" t="n"/>
+      <c r="J8" s="23" t="inlineStr"/>
+      <c r="K8" s="25" t="n"/>
+      <c r="L8" s="25" t="n"/>
+      <c r="M8" s="25" t="n"/>
+      <c r="N8" s="25" t="n"/>
+      <c r="O8" s="25" t="n"/>
     </row>
     <row r="9" ht="39" customHeight="1">
       <c r="B9" s="11" t="inlineStr">
@@ -2009,7 +2402,7 @@
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr"/>
-      <c r="D9" s="25" t="inlineStr">
+      <c r="D9" s="26" t="inlineStr">
         <is>
           <t>Impact Accelerators</t>
         </is>
@@ -2019,10 +2412,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F9" s="26" t="n"/>
-      <c r="G9" s="26" t="n"/>
-      <c r="H9" s="26" t="n"/>
-      <c r="I9" s="26" t="n"/>
+      <c r="F9" s="27" t="n"/>
+      <c r="G9" s="27" t="n"/>
+      <c r="H9" s="27" t="n"/>
+      <c r="I9" s="27" t="n"/>
       <c r="J9" s="13" t="inlineStr">
         <is>
           <t>New – no data yet</t>
@@ -2041,7 +2434,7 @@
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr"/>
-      <c r="D10" s="25" t="inlineStr">
+      <c r="D10" s="26" t="inlineStr">
         <is>
           <t>Strategic Initiatives 2</t>
         </is>
@@ -2051,10 +2444,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F10" s="26" t="n"/>
-      <c r="G10" s="26" t="n"/>
-      <c r="H10" s="26" t="n"/>
-      <c r="I10" s="26" t="n"/>
+      <c r="F10" s="27" t="n"/>
+      <c r="G10" s="27" t="n"/>
+      <c r="H10" s="27" t="n"/>
+      <c r="I10" s="27" t="n"/>
       <c r="J10" s="13" t="inlineStr">
         <is>
           <t>New – no data yet</t>
@@ -2073,7 +2466,7 @@
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr"/>
-      <c r="D11" s="25" t="inlineStr">
+      <c r="D11" s="26" t="inlineStr">
         <is>
           <t>Strategic Initiatives 3</t>
         </is>
@@ -2083,10 +2476,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F11" s="26" t="n"/>
-      <c r="G11" s="26" t="n"/>
-      <c r="H11" s="26" t="n"/>
-      <c r="I11" s="26" t="n"/>
+      <c r="F11" s="27" t="n"/>
+      <c r="G11" s="27" t="n"/>
+      <c r="H11" s="27" t="n"/>
+      <c r="I11" s="27" t="n"/>
       <c r="J11" s="13" t="inlineStr">
         <is>
           <t>New – no data yet</t>
@@ -2115,10 +2508,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F12" s="26" t="n"/>
-      <c r="G12" s="26" t="n"/>
-      <c r="H12" s="26" t="n"/>
-      <c r="I12" s="26" t="n"/>
+      <c r="F12" s="27" t="n"/>
+      <c r="G12" s="27" t="n"/>
+      <c r="H12" s="27" t="n"/>
+      <c r="I12" s="27" t="n"/>
       <c r="J12" s="13" t="inlineStr">
         <is>
           <t>New – no data yet</t>
@@ -2147,10 +2540,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F13" s="26" t="n"/>
-      <c r="G13" s="26" t="n"/>
-      <c r="H13" s="26" t="n"/>
-      <c r="I13" s="26" t="n"/>
+      <c r="F13" s="27" t="n"/>
+      <c r="G13" s="27" t="n"/>
+      <c r="H13" s="27" t="n"/>
+      <c r="I13" s="27" t="n"/>
       <c r="J13" s="13" t="inlineStr">
         <is>
           <t>New – no data yet</t>
@@ -2163,32 +2556,32 @@
       <c r="O13" s="13" t="n"/>
     </row>
     <row r="14" ht="88" customHeight="1">
-      <c r="B14" s="22" t="inlineStr">
-        <is>
-          <t>TR2(c)</t>
-        </is>
-      </c>
-      <c r="C14" s="22" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>TR2(c)</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>Expert-reviewed summary of sustainability-related research outputs, outcomes and influence using available institutional evidence sources</t>
         </is>
       </c>
-      <c r="D14" s="22" t="inlineStr">
+      <c r="D14" s="23" t="inlineStr">
         <is>
           <t>SDG-related research outputs in the top 10% of citations</t>
         </is>
       </c>
-      <c r="E14" s="22" t="inlineStr"/>
-      <c r="F14" s="23" t="n"/>
-      <c r="G14" s="23" t="n"/>
-      <c r="H14" s="23" t="n"/>
-      <c r="I14" s="23" t="n"/>
-      <c r="J14" s="22" t="inlineStr"/>
-      <c r="K14" s="24" t="n"/>
-      <c r="L14" s="24" t="n"/>
-      <c r="M14" s="24" t="n"/>
-      <c r="N14" s="24" t="n"/>
-      <c r="O14" s="24" t="n"/>
+      <c r="E14" s="23" t="inlineStr"/>
+      <c r="F14" s="24" t="n"/>
+      <c r="G14" s="24" t="n"/>
+      <c r="H14" s="24" t="n"/>
+      <c r="I14" s="24" t="n"/>
+      <c r="J14" s="23" t="inlineStr"/>
+      <c r="K14" s="25" t="n"/>
+      <c r="L14" s="25" t="n"/>
+      <c r="M14" s="25" t="n"/>
+      <c r="N14" s="25" t="n"/>
+      <c r="O14" s="25" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="11" t="inlineStr">
@@ -2197,7 +2590,7 @@
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr"/>
-      <c r="D15" s="25" t="inlineStr">
+      <c r="D15" s="26" t="inlineStr">
         <is>
           <t>SDG 1 - No Poverty</t>
         </is>
@@ -2207,10 +2600,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F15" s="26" t="n"/>
-      <c r="G15" s="26" t="n"/>
-      <c r="H15" s="26" t="n"/>
-      <c r="I15" s="26" t="n">
+      <c r="F15" s="27" t="n"/>
+      <c r="G15" s="27" t="n"/>
+      <c r="H15" s="27" t="n"/>
+      <c r="I15" s="27" t="n">
         <v>424</v>
       </c>
       <c r="J15" s="13" t="inlineStr">
@@ -2231,7 +2624,7 @@
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr"/>
-      <c r="D16" s="25" t="inlineStr">
+      <c r="D16" s="26" t="inlineStr">
         <is>
           <t>SDG 2 - Zero Hunger</t>
         </is>
@@ -2241,10 +2634,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F16" s="26" t="n"/>
-      <c r="G16" s="26" t="n"/>
-      <c r="H16" s="26" t="n"/>
-      <c r="I16" s="26" t="n">
+      <c r="F16" s="27" t="n"/>
+      <c r="G16" s="27" t="n"/>
+      <c r="H16" s="27" t="n"/>
+      <c r="I16" s="27" t="n">
         <v>781</v>
       </c>
       <c r="J16" s="13" t="inlineStr">
@@ -2265,7 +2658,7 @@
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr"/>
-      <c r="D17" s="25" t="inlineStr">
+      <c r="D17" s="26" t="inlineStr">
         <is>
           <t>SDG 3 - Good health and well-being</t>
         </is>
@@ -2275,10 +2668,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F17" s="26" t="n"/>
-      <c r="G17" s="26" t="n"/>
-      <c r="H17" s="26" t="n"/>
-      <c r="I17" s="26" t="n">
+      <c r="F17" s="27" t="n"/>
+      <c r="G17" s="27" t="n"/>
+      <c r="H17" s="27" t="n"/>
+      <c r="I17" s="27" t="n">
         <v>15195</v>
       </c>
       <c r="J17" s="13" t="inlineStr">
@@ -2299,7 +2692,7 @@
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr"/>
-      <c r="D18" s="25" t="inlineStr">
+      <c r="D18" s="26" t="inlineStr">
         <is>
           <t>SDG 4 - Quality Education</t>
         </is>
@@ -2309,10 +2702,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F18" s="26" t="n"/>
-      <c r="G18" s="26" t="n"/>
-      <c r="H18" s="26" t="n"/>
-      <c r="I18" s="26" t="n">
+      <c r="F18" s="27" t="n"/>
+      <c r="G18" s="27" t="n"/>
+      <c r="H18" s="27" t="n"/>
+      <c r="I18" s="27" t="n">
         <v>1292</v>
       </c>
       <c r="J18" s="13" t="inlineStr">
@@ -2333,7 +2726,7 @@
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr"/>
-      <c r="D19" s="25" t="inlineStr">
+      <c r="D19" s="26" t="inlineStr">
         <is>
           <t>SDG 5 - Gender Equality</t>
         </is>
@@ -2343,10 +2736,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F19" s="26" t="n"/>
-      <c r="G19" s="26" t="n"/>
-      <c r="H19" s="26" t="n"/>
-      <c r="I19" s="26" t="n">
+      <c r="F19" s="27" t="n"/>
+      <c r="G19" s="27" t="n"/>
+      <c r="H19" s="27" t="n"/>
+      <c r="I19" s="27" t="n">
         <v>1275</v>
       </c>
       <c r="J19" s="13" t="inlineStr">
@@ -2367,7 +2760,7 @@
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr"/>
-      <c r="D20" s="25" t="inlineStr">
+      <c r="D20" s="26" t="inlineStr">
         <is>
           <t>SDG 6 - Clean water and sanitation</t>
         </is>
@@ -2377,10 +2770,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F20" s="26" t="n"/>
-      <c r="G20" s="26" t="n"/>
-      <c r="H20" s="26" t="n"/>
-      <c r="I20" s="26" t="n">
+      <c r="F20" s="27" t="n"/>
+      <c r="G20" s="27" t="n"/>
+      <c r="H20" s="27" t="n"/>
+      <c r="I20" s="27" t="n">
         <v>661</v>
       </c>
       <c r="J20" s="13" t="inlineStr">
@@ -2401,7 +2794,7 @@
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr"/>
-      <c r="D21" s="25" t="inlineStr">
+      <c r="D21" s="26" t="inlineStr">
         <is>
           <t>SDG 7 - Affordable and clean energy</t>
         </is>
@@ -2411,10 +2804,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F21" s="26" t="n"/>
-      <c r="G21" s="26" t="n"/>
-      <c r="H21" s="26" t="n"/>
-      <c r="I21" s="26" t="n">
+      <c r="F21" s="27" t="n"/>
+      <c r="G21" s="27" t="n"/>
+      <c r="H21" s="27" t="n"/>
+      <c r="I21" s="27" t="n">
         <v>997</v>
       </c>
       <c r="J21" s="13" t="inlineStr">
@@ -2435,7 +2828,7 @@
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr"/>
-      <c r="D22" s="25" t="inlineStr">
+      <c r="D22" s="26" t="inlineStr">
         <is>
           <t>SDG 8 - Decent work and economic growth</t>
         </is>
@@ -2445,10 +2838,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F22" s="26" t="n"/>
-      <c r="G22" s="26" t="n"/>
-      <c r="H22" s="26" t="n"/>
-      <c r="I22" s="26" t="n">
+      <c r="F22" s="27" t="n"/>
+      <c r="G22" s="27" t="n"/>
+      <c r="H22" s="27" t="n"/>
+      <c r="I22" s="27" t="n">
         <v>995</v>
       </c>
       <c r="J22" s="13" t="inlineStr">
@@ -2469,7 +2862,7 @@
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr"/>
-      <c r="D23" s="25" t="inlineStr">
+      <c r="D23" s="26" t="inlineStr">
         <is>
           <t>SDG 9 - Industry, innovation and infrastructure</t>
         </is>
@@ -2479,10 +2872,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F23" s="26" t="n"/>
-      <c r="G23" s="26" t="n"/>
-      <c r="H23" s="26" t="n"/>
-      <c r="I23" s="26" t="n">
+      <c r="F23" s="27" t="n"/>
+      <c r="G23" s="27" t="n"/>
+      <c r="H23" s="27" t="n"/>
+      <c r="I23" s="27" t="n">
         <v>1457</v>
       </c>
       <c r="J23" s="13" t="inlineStr">
@@ -2503,7 +2896,7 @@
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr"/>
-      <c r="D24" s="25" t="inlineStr">
+      <c r="D24" s="26" t="inlineStr">
         <is>
           <t>SDG 10 - Reduced inequality</t>
         </is>
@@ -2513,10 +2906,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F24" s="26" t="n"/>
-      <c r="G24" s="26" t="n"/>
-      <c r="H24" s="26" t="n"/>
-      <c r="I24" s="26" t="n">
+      <c r="F24" s="27" t="n"/>
+      <c r="G24" s="27" t="n"/>
+      <c r="H24" s="27" t="n"/>
+      <c r="I24" s="27" t="n">
         <v>1617</v>
       </c>
       <c r="J24" s="13" t="inlineStr">
@@ -2537,7 +2930,7 @@
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr"/>
-      <c r="D25" s="25" t="inlineStr">
+      <c r="D25" s="26" t="inlineStr">
         <is>
           <t>SDG 11 - Sustainable cities and communities</t>
         </is>
@@ -2547,10 +2940,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F25" s="26" t="n"/>
-      <c r="G25" s="26" t="n"/>
-      <c r="H25" s="26" t="n"/>
-      <c r="I25" s="26" t="n">
+      <c r="F25" s="27" t="n"/>
+      <c r="G25" s="27" t="n"/>
+      <c r="H25" s="27" t="n"/>
+      <c r="I25" s="27" t="n">
         <v>1436</v>
       </c>
       <c r="J25" s="13" t="inlineStr">
@@ -2571,7 +2964,7 @@
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr"/>
-      <c r="D26" s="25" t="inlineStr">
+      <c r="D26" s="26" t="inlineStr">
         <is>
           <t>SDG 12 - Responsible consumption and production</t>
         </is>
@@ -2581,10 +2974,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F26" s="26" t="n"/>
-      <c r="G26" s="26" t="n"/>
-      <c r="H26" s="26" t="n"/>
-      <c r="I26" s="26" t="n">
+      <c r="F26" s="27" t="n"/>
+      <c r="G26" s="27" t="n"/>
+      <c r="H26" s="27" t="n"/>
+      <c r="I26" s="27" t="n">
         <v>838</v>
       </c>
       <c r="J26" s="13" t="inlineStr">
@@ -2605,7 +2998,7 @@
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr"/>
-      <c r="D27" s="25" t="inlineStr">
+      <c r="D27" s="26" t="inlineStr">
         <is>
           <t>SDG 13 - Climate action</t>
         </is>
@@ -2615,10 +3008,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F27" s="26" t="n"/>
-      <c r="G27" s="26" t="n"/>
-      <c r="H27" s="26" t="n"/>
-      <c r="I27" s="26" t="n">
+      <c r="F27" s="27" t="n"/>
+      <c r="G27" s="27" t="n"/>
+      <c r="H27" s="27" t="n"/>
+      <c r="I27" s="27" t="n">
         <v>1624</v>
       </c>
       <c r="J27" s="13" t="inlineStr">
@@ -2639,7 +3032,7 @@
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr"/>
-      <c r="D28" s="25" t="inlineStr">
+      <c r="D28" s="26" t="inlineStr">
         <is>
           <t>SDG 14 - Life below water</t>
         </is>
@@ -2649,10 +3042,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F28" s="26" t="n"/>
-      <c r="G28" s="26" t="n"/>
-      <c r="H28" s="26" t="n"/>
-      <c r="I28" s="26" t="n">
+      <c r="F28" s="27" t="n"/>
+      <c r="G28" s="27" t="n"/>
+      <c r="H28" s="27" t="n"/>
+      <c r="I28" s="27" t="n">
         <v>442</v>
       </c>
       <c r="J28" s="13" t="inlineStr">
@@ -2673,7 +3066,7 @@
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr"/>
-      <c r="D29" s="25" t="inlineStr">
+      <c r="D29" s="26" t="inlineStr">
         <is>
           <t>SDG 15 - Life on land</t>
         </is>
@@ -2683,10 +3076,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F29" s="26" t="n"/>
-      <c r="G29" s="26" t="n"/>
-      <c r="H29" s="26" t="n"/>
-      <c r="I29" s="26" t="n">
+      <c r="F29" s="27" t="n"/>
+      <c r="G29" s="27" t="n"/>
+      <c r="H29" s="27" t="n"/>
+      <c r="I29" s="27" t="n">
         <v>1015</v>
       </c>
       <c r="J29" s="13" t="inlineStr">
@@ -2707,7 +3100,7 @@
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr"/>
-      <c r="D30" s="25" t="inlineStr">
+      <c r="D30" s="26" t="inlineStr">
         <is>
           <t>SDG 16 - Peace, justice and strong institutions</t>
         </is>
@@ -2717,10 +3110,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F30" s="26" t="n"/>
-      <c r="G30" s="26" t="n"/>
-      <c r="H30" s="26" t="n"/>
-      <c r="I30" s="26" t="n">
+      <c r="F30" s="27" t="n"/>
+      <c r="G30" s="27" t="n"/>
+      <c r="H30" s="27" t="n"/>
+      <c r="I30" s="27" t="n">
         <v>1681</v>
       </c>
       <c r="J30" s="13" t="inlineStr">
@@ -2735,28 +3128,28 @@
       <c r="O30" s="13" t="n"/>
     </row>
     <row r="31" ht="39" customHeight="1">
-      <c r="B31" s="22" t="inlineStr">
-        <is>
-          <t>TR2(c)</t>
-        </is>
-      </c>
-      <c r="C31" s="22" t="inlineStr"/>
-      <c r="D31" s="22" t="inlineStr">
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>TR2(c)</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="inlineStr"/>
+      <c r="D31" s="23" t="inlineStr">
         <is>
           <t>SDG-related research outputs in the top 10% of citations (Field-weighted)</t>
         </is>
       </c>
-      <c r="E31" s="22" t="inlineStr"/>
-      <c r="F31" s="23" t="n"/>
-      <c r="G31" s="23" t="n"/>
-      <c r="H31" s="23" t="n"/>
-      <c r="I31" s="23" t="n"/>
-      <c r="J31" s="22" t="inlineStr"/>
-      <c r="K31" s="24" t="n"/>
-      <c r="L31" s="24" t="n"/>
-      <c r="M31" s="24" t="n"/>
-      <c r="N31" s="24" t="n"/>
-      <c r="O31" s="24" t="n"/>
+      <c r="E31" s="23" t="inlineStr"/>
+      <c r="F31" s="24" t="n"/>
+      <c r="G31" s="24" t="n"/>
+      <c r="H31" s="24" t="n"/>
+      <c r="I31" s="24" t="n"/>
+      <c r="J31" s="23" t="inlineStr"/>
+      <c r="K31" s="25" t="n"/>
+      <c r="L31" s="25" t="n"/>
+      <c r="M31" s="25" t="n"/>
+      <c r="N31" s="25" t="n"/>
+      <c r="O31" s="25" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="B32" s="11" t="inlineStr">
@@ -2765,7 +3158,7 @@
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr"/>
-      <c r="D32" s="25" t="inlineStr">
+      <c r="D32" s="26" t="inlineStr">
         <is>
           <t>SDG 1 - No Poverty</t>
         </is>
@@ -2775,10 +3168,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F32" s="26" t="n"/>
-      <c r="G32" s="26" t="n"/>
-      <c r="H32" s="26" t="n"/>
-      <c r="I32" s="26" t="n">
+      <c r="F32" s="27" t="n"/>
+      <c r="G32" s="27" t="n"/>
+      <c r="H32" s="27" t="n"/>
+      <c r="I32" s="27" t="n">
         <v>20</v>
       </c>
       <c r="J32" s="13" t="inlineStr">
@@ -2799,7 +3192,7 @@
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr"/>
-      <c r="D33" s="25" t="inlineStr">
+      <c r="D33" s="26" t="inlineStr">
         <is>
           <t>SDG 2 - Zero Hunger</t>
         </is>
@@ -2809,10 +3202,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F33" s="26" t="n"/>
-      <c r="G33" s="26" t="n"/>
-      <c r="H33" s="26" t="n"/>
-      <c r="I33" s="26" t="n">
+      <c r="F33" s="27" t="n"/>
+      <c r="G33" s="27" t="n"/>
+      <c r="H33" s="27" t="n"/>
+      <c r="I33" s="27" t="n">
         <v>19</v>
       </c>
       <c r="J33" s="13" t="inlineStr">
@@ -2833,7 +3226,7 @@
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr"/>
-      <c r="D34" s="25" t="inlineStr">
+      <c r="D34" s="26" t="inlineStr">
         <is>
           <t>SDG 3 - Good health and well-being</t>
         </is>
@@ -2843,10 +3236,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F34" s="26" t="n"/>
-      <c r="G34" s="26" t="n"/>
-      <c r="H34" s="26" t="n"/>
-      <c r="I34" s="26" t="n">
+      <c r="F34" s="27" t="n"/>
+      <c r="G34" s="27" t="n"/>
+      <c r="H34" s="27" t="n"/>
+      <c r="I34" s="27" t="n">
         <v>20</v>
       </c>
       <c r="J34" s="13" t="inlineStr">
@@ -2867,7 +3260,7 @@
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr"/>
-      <c r="D35" s="25" t="inlineStr">
+      <c r="D35" s="26" t="inlineStr">
         <is>
           <t>SDG 4 - Quality Education</t>
         </is>
@@ -2877,10 +3270,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F35" s="26" t="n"/>
-      <c r="G35" s="26" t="n"/>
-      <c r="H35" s="26" t="n"/>
-      <c r="I35" s="26" t="n">
+      <c r="F35" s="27" t="n"/>
+      <c r="G35" s="27" t="n"/>
+      <c r="H35" s="27" t="n"/>
+      <c r="I35" s="27" t="n">
         <v>19</v>
       </c>
       <c r="J35" s="13" t="inlineStr">
@@ -2901,7 +3294,7 @@
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr"/>
-      <c r="D36" s="25" t="inlineStr">
+      <c r="D36" s="26" t="inlineStr">
         <is>
           <t>SDG 5 - Gender Equality</t>
         </is>
@@ -2911,10 +3304,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F36" s="26" t="n"/>
-      <c r="G36" s="26" t="n"/>
-      <c r="H36" s="26" t="n"/>
-      <c r="I36" s="26" t="n">
+      <c r="F36" s="27" t="n"/>
+      <c r="G36" s="27" t="n"/>
+      <c r="H36" s="27" t="n"/>
+      <c r="I36" s="27" t="n">
         <v>18</v>
       </c>
       <c r="J36" s="13" t="inlineStr">
@@ -2935,7 +3328,7 @@
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr"/>
-      <c r="D37" s="25" t="inlineStr">
+      <c r="D37" s="26" t="inlineStr">
         <is>
           <t>SDG 6 - Clean water and sanitation</t>
         </is>
@@ -2945,10 +3338,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F37" s="26" t="n"/>
-      <c r="G37" s="26" t="n"/>
-      <c r="H37" s="26" t="n"/>
-      <c r="I37" s="26" t="n">
+      <c r="F37" s="27" t="n"/>
+      <c r="G37" s="27" t="n"/>
+      <c r="H37" s="27" t="n"/>
+      <c r="I37" s="27" t="n">
         <v>17</v>
       </c>
       <c r="J37" s="13" t="inlineStr">
@@ -2969,7 +3362,7 @@
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr"/>
-      <c r="D38" s="25" t="inlineStr">
+      <c r="D38" s="26" t="inlineStr">
         <is>
           <t>SDG 7 - Affordable and clean energy</t>
         </is>
@@ -2979,10 +3372,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F38" s="26" t="n"/>
-      <c r="G38" s="26" t="n"/>
-      <c r="H38" s="26" t="n"/>
-      <c r="I38" s="26" t="n">
+      <c r="F38" s="27" t="n"/>
+      <c r="G38" s="27" t="n"/>
+      <c r="H38" s="27" t="n"/>
+      <c r="I38" s="27" t="n">
         <v>22</v>
       </c>
       <c r="J38" s="13" t="inlineStr">
@@ -3003,7 +3396,7 @@
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr"/>
-      <c r="D39" s="25" t="inlineStr">
+      <c r="D39" s="26" t="inlineStr">
         <is>
           <t>SDG 8 - Decent work and economic growth</t>
         </is>
@@ -3013,10 +3406,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F39" s="26" t="n"/>
-      <c r="G39" s="26" t="n"/>
-      <c r="H39" s="26" t="n"/>
-      <c r="I39" s="26" t="n">
+      <c r="F39" s="27" t="n"/>
+      <c r="G39" s="27" t="n"/>
+      <c r="H39" s="27" t="n"/>
+      <c r="I39" s="27" t="n">
         <v>22</v>
       </c>
       <c r="J39" s="13" t="inlineStr">
@@ -3037,7 +3430,7 @@
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr"/>
-      <c r="D40" s="25" t="inlineStr">
+      <c r="D40" s="26" t="inlineStr">
         <is>
           <t>SDG 9 - Industry, innovation and infrastructure</t>
         </is>
@@ -3047,10 +3440,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F40" s="26" t="n"/>
-      <c r="G40" s="26" t="n"/>
-      <c r="H40" s="26" t="n"/>
-      <c r="I40" s="26" t="n">
+      <c r="F40" s="27" t="n"/>
+      <c r="G40" s="27" t="n"/>
+      <c r="H40" s="27" t="n"/>
+      <c r="I40" s="27" t="n">
         <v>23</v>
       </c>
       <c r="J40" s="13" t="inlineStr">
@@ -3071,7 +3464,7 @@
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr"/>
-      <c r="D41" s="25" t="inlineStr">
+      <c r="D41" s="26" t="inlineStr">
         <is>
           <t>SDG 10 - Reduced inequality</t>
         </is>
@@ -3081,10 +3474,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F41" s="26" t="n"/>
-      <c r="G41" s="26" t="n"/>
-      <c r="H41" s="26" t="n"/>
-      <c r="I41" s="26" t="n">
+      <c r="F41" s="27" t="n"/>
+      <c r="G41" s="27" t="n"/>
+      <c r="H41" s="27" t="n"/>
+      <c r="I41" s="27" t="n">
         <v>20</v>
       </c>
       <c r="J41" s="13" t="inlineStr">
@@ -3105,7 +3498,7 @@
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr"/>
-      <c r="D42" s="25" t="inlineStr">
+      <c r="D42" s="26" t="inlineStr">
         <is>
           <t>SDG 11 - Sustainable cities and communities</t>
         </is>
@@ -3115,10 +3508,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F42" s="26" t="n"/>
-      <c r="G42" s="26" t="n"/>
-      <c r="H42" s="26" t="n"/>
-      <c r="I42" s="26" t="n">
+      <c r="F42" s="27" t="n"/>
+      <c r="G42" s="27" t="n"/>
+      <c r="H42" s="27" t="n"/>
+      <c r="I42" s="27" t="n">
         <v>20</v>
       </c>
       <c r="J42" s="13" t="inlineStr">
@@ -3139,7 +3532,7 @@
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr"/>
-      <c r="D43" s="25" t="inlineStr">
+      <c r="D43" s="26" t="inlineStr">
         <is>
           <t>SDG 12 - Responsible consumption and production</t>
         </is>
@@ -3149,10 +3542,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F43" s="26" t="n"/>
-      <c r="G43" s="26" t="n"/>
-      <c r="H43" s="26" t="n"/>
-      <c r="I43" s="26" t="n">
+      <c r="F43" s="27" t="n"/>
+      <c r="G43" s="27" t="n"/>
+      <c r="H43" s="27" t="n"/>
+      <c r="I43" s="27" t="n">
         <v>20</v>
       </c>
       <c r="J43" s="13" t="inlineStr">
@@ -3173,7 +3566,7 @@
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr"/>
-      <c r="D44" s="25" t="inlineStr">
+      <c r="D44" s="26" t="inlineStr">
         <is>
           <t>SDG 13 - Climate action</t>
         </is>
@@ -3183,10 +3576,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F44" s="26" t="n"/>
-      <c r="G44" s="26" t="n"/>
-      <c r="H44" s="26" t="n"/>
-      <c r="I44" s="26" t="n">
+      <c r="F44" s="27" t="n"/>
+      <c r="G44" s="27" t="n"/>
+      <c r="H44" s="27" t="n"/>
+      <c r="I44" s="27" t="n">
         <v>26</v>
       </c>
       <c r="J44" s="13" t="inlineStr">
@@ -3207,7 +3600,7 @@
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr"/>
-      <c r="D45" s="25" t="inlineStr">
+      <c r="D45" s="26" t="inlineStr">
         <is>
           <t>SDG 14 - Life below water</t>
         </is>
@@ -3217,10 +3610,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F45" s="26" t="n"/>
-      <c r="G45" s="26" t="n"/>
-      <c r="H45" s="26" t="n"/>
-      <c r="I45" s="26" t="n">
+      <c r="F45" s="27" t="n"/>
+      <c r="G45" s="27" t="n"/>
+      <c r="H45" s="27" t="n"/>
+      <c r="I45" s="27" t="n">
         <v>20</v>
       </c>
       <c r="J45" s="13" t="inlineStr">
@@ -3241,7 +3634,7 @@
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr"/>
-      <c r="D46" s="25" t="inlineStr">
+      <c r="D46" s="26" t="inlineStr">
         <is>
           <t>SDG 15 - Life on land</t>
         </is>
@@ -3251,10 +3644,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F46" s="26" t="n"/>
-      <c r="G46" s="26" t="n"/>
-      <c r="H46" s="26" t="n"/>
-      <c r="I46" s="26" t="n">
+      <c r="F46" s="27" t="n"/>
+      <c r="G46" s="27" t="n"/>
+      <c r="H46" s="27" t="n"/>
+      <c r="I46" s="27" t="n">
         <v>17</v>
       </c>
       <c r="J46" s="13" t="inlineStr">
@@ -3275,7 +3668,7 @@
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr"/>
-      <c r="D47" s="25" t="inlineStr">
+      <c r="D47" s="26" t="inlineStr">
         <is>
           <t>SDG 16 - Peace, justice and strong institutions</t>
         </is>
@@ -3285,10 +3678,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F47" s="26" t="n"/>
-      <c r="G47" s="26" t="n"/>
-      <c r="H47" s="26" t="n"/>
-      <c r="I47" s="26" t="n">
+      <c r="F47" s="27" t="n"/>
+      <c r="G47" s="27" t="n"/>
+      <c r="H47" s="27" t="n"/>
+      <c r="I47" s="27" t="n">
         <v>20</v>
       </c>
       <c r="J47" s="13" t="inlineStr">
@@ -3319,10 +3712,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F48" s="26" t="n"/>
-      <c r="G48" s="26" t="n"/>
-      <c r="H48" s="26" t="n"/>
-      <c r="I48" s="26" t="n">
+      <c r="F48" s="27" t="n"/>
+      <c r="G48" s="27" t="n"/>
+      <c r="H48" s="27" t="n"/>
+      <c r="I48" s="27" t="n">
         <v>651</v>
       </c>
       <c r="J48" s="13" t="inlineStr">
@@ -3343,7 +3736,7 @@
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr"/>
-      <c r="D49" s="25" t="inlineStr">
+      <c r="D49" s="26" t="inlineStr">
         <is>
           <t>SDG 1 - No Poverty</t>
         </is>
@@ -3353,10 +3746,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F49" s="26" t="n"/>
-      <c r="G49" s="26" t="n"/>
-      <c r="H49" s="26" t="n"/>
-      <c r="I49" s="26" t="n">
+      <c r="F49" s="27" t="n"/>
+      <c r="G49" s="27" t="n"/>
+      <c r="H49" s="27" t="n"/>
+      <c r="I49" s="27" t="n">
         <v>0</v>
       </c>
       <c r="J49" s="13" t="inlineStr">
@@ -3377,7 +3770,7 @@
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr"/>
-      <c r="D50" s="25" t="inlineStr">
+      <c r="D50" s="26" t="inlineStr">
         <is>
           <t>SDG 2 - Zero Hunger</t>
         </is>
@@ -3387,10 +3780,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F50" s="26" t="n"/>
-      <c r="G50" s="26" t="n"/>
-      <c r="H50" s="26" t="n"/>
-      <c r="I50" s="26" t="n">
+      <c r="F50" s="27" t="n"/>
+      <c r="G50" s="27" t="n"/>
+      <c r="H50" s="27" t="n"/>
+      <c r="I50" s="27" t="n">
         <v>6</v>
       </c>
       <c r="J50" s="13" t="inlineStr">
@@ -3411,7 +3804,7 @@
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr"/>
-      <c r="D51" s="25" t="inlineStr">
+      <c r="D51" s="26" t="inlineStr">
         <is>
           <t>SDG 3 - Good health and well-being</t>
         </is>
@@ -3421,10 +3814,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F51" s="26" t="n"/>
-      <c r="G51" s="26" t="n"/>
-      <c r="H51" s="26" t="n"/>
-      <c r="I51" s="26" t="n">
+      <c r="F51" s="27" t="n"/>
+      <c r="G51" s="27" t="n"/>
+      <c r="H51" s="27" t="n"/>
+      <c r="I51" s="27" t="n">
         <v>564</v>
       </c>
       <c r="J51" s="13" t="inlineStr">
@@ -3445,7 +3838,7 @@
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr"/>
-      <c r="D52" s="25" t="inlineStr">
+      <c r="D52" s="26" t="inlineStr">
         <is>
           <t>SDG 4 - Quality Education</t>
         </is>
@@ -3455,10 +3848,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F52" s="26" t="n"/>
-      <c r="G52" s="26" t="n"/>
-      <c r="H52" s="26" t="n"/>
-      <c r="I52" s="26" t="n">
+      <c r="F52" s="27" t="n"/>
+      <c r="G52" s="27" t="n"/>
+      <c r="H52" s="27" t="n"/>
+      <c r="I52" s="27" t="n">
         <v>7</v>
       </c>
       <c r="J52" s="13" t="inlineStr">
@@ -3479,7 +3872,7 @@
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr"/>
-      <c r="D53" s="25" t="inlineStr">
+      <c r="D53" s="26" t="inlineStr">
         <is>
           <t>SDG 5 - Gender Equality</t>
         </is>
@@ -3489,10 +3882,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F53" s="26" t="n"/>
-      <c r="G53" s="26" t="n"/>
-      <c r="H53" s="26" t="n"/>
-      <c r="I53" s="26" t="n">
+      <c r="F53" s="27" t="n"/>
+      <c r="G53" s="27" t="n"/>
+      <c r="H53" s="27" t="n"/>
+      <c r="I53" s="27" t="n">
         <v>0</v>
       </c>
       <c r="J53" s="13" t="inlineStr">
@@ -3513,7 +3906,7 @@
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr"/>
-      <c r="D54" s="25" t="inlineStr">
+      <c r="D54" s="26" t="inlineStr">
         <is>
           <t>SDG 6 - Clean water and sanitation</t>
         </is>
@@ -3523,10 +3916,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F54" s="26" t="n"/>
-      <c r="G54" s="26" t="n"/>
-      <c r="H54" s="26" t="n"/>
-      <c r="I54" s="26" t="n">
+      <c r="F54" s="27" t="n"/>
+      <c r="G54" s="27" t="n"/>
+      <c r="H54" s="27" t="n"/>
+      <c r="I54" s="27" t="n">
         <v>1</v>
       </c>
       <c r="J54" s="13" t="inlineStr">
@@ -3547,7 +3940,7 @@
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr"/>
-      <c r="D55" s="25" t="inlineStr">
+      <c r="D55" s="26" t="inlineStr">
         <is>
           <t>SDG 7 - Affordable and clean energy</t>
         </is>
@@ -3557,10 +3950,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F55" s="26" t="n"/>
-      <c r="G55" s="26" t="n"/>
-      <c r="H55" s="26" t="n"/>
-      <c r="I55" s="26" t="n">
+      <c r="F55" s="27" t="n"/>
+      <c r="G55" s="27" t="n"/>
+      <c r="H55" s="27" t="n"/>
+      <c r="I55" s="27" t="n">
         <v>34</v>
       </c>
       <c r="J55" s="13" t="inlineStr">
@@ -3581,7 +3974,7 @@
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr"/>
-      <c r="D56" s="25" t="inlineStr">
+      <c r="D56" s="26" t="inlineStr">
         <is>
           <t>SDG 8 - Decent work and economic growth</t>
         </is>
@@ -3591,10 +3984,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F56" s="26" t="n"/>
-      <c r="G56" s="26" t="n"/>
-      <c r="H56" s="26" t="n"/>
-      <c r="I56" s="26" t="n">
+      <c r="F56" s="27" t="n"/>
+      <c r="G56" s="27" t="n"/>
+      <c r="H56" s="27" t="n"/>
+      <c r="I56" s="27" t="n">
         <v>0</v>
       </c>
       <c r="J56" s="13" t="inlineStr">
@@ -3615,7 +4008,7 @@
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr"/>
-      <c r="D57" s="25" t="inlineStr">
+      <c r="D57" s="26" t="inlineStr">
         <is>
           <t>SDG 9 - Industry, innovation and infrastructure</t>
         </is>
@@ -3625,10 +4018,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F57" s="26" t="n"/>
-      <c r="G57" s="26" t="n"/>
-      <c r="H57" s="26" t="n"/>
-      <c r="I57" s="26" t="n">
+      <c r="F57" s="27" t="n"/>
+      <c r="G57" s="27" t="n"/>
+      <c r="H57" s="27" t="n"/>
+      <c r="I57" s="27" t="n">
         <v>1</v>
       </c>
       <c r="J57" s="13" t="inlineStr">
@@ -3649,7 +4042,7 @@
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr"/>
-      <c r="D58" s="25" t="inlineStr">
+      <c r="D58" s="26" t="inlineStr">
         <is>
           <t>SDG 10 - Reduced inequality</t>
         </is>
@@ -3659,10 +4052,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F58" s="26" t="n"/>
-      <c r="G58" s="26" t="n"/>
-      <c r="H58" s="26" t="n"/>
-      <c r="I58" s="26" t="n">
+      <c r="F58" s="27" t="n"/>
+      <c r="G58" s="27" t="n"/>
+      <c r="H58" s="27" t="n"/>
+      <c r="I58" s="27" t="n">
         <v>1</v>
       </c>
       <c r="J58" s="13" t="inlineStr">
@@ -3683,7 +4076,7 @@
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr"/>
-      <c r="D59" s="25" t="inlineStr">
+      <c r="D59" s="26" t="inlineStr">
         <is>
           <t>SDG 11 - Sustainable cities and communities</t>
         </is>
@@ -3693,10 +4086,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F59" s="26" t="n"/>
-      <c r="G59" s="26" t="n"/>
-      <c r="H59" s="26" t="n"/>
-      <c r="I59" s="26" t="n">
+      <c r="F59" s="27" t="n"/>
+      <c r="G59" s="27" t="n"/>
+      <c r="H59" s="27" t="n"/>
+      <c r="I59" s="27" t="n">
         <v>6</v>
       </c>
       <c r="J59" s="13" t="inlineStr">
@@ -3717,7 +4110,7 @@
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr"/>
-      <c r="D60" s="25" t="inlineStr">
+      <c r="D60" s="26" t="inlineStr">
         <is>
           <t>SDG 12 - Responsible consumption and production</t>
         </is>
@@ -3727,10 +4120,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F60" s="26" t="n"/>
-      <c r="G60" s="26" t="n"/>
-      <c r="H60" s="26" t="n"/>
-      <c r="I60" s="26" t="n">
+      <c r="F60" s="27" t="n"/>
+      <c r="G60" s="27" t="n"/>
+      <c r="H60" s="27" t="n"/>
+      <c r="I60" s="27" t="n">
         <v>8</v>
       </c>
       <c r="J60" s="13" t="inlineStr">
@@ -3751,7 +4144,7 @@
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr"/>
-      <c r="D61" s="25" t="inlineStr">
+      <c r="D61" s="26" t="inlineStr">
         <is>
           <t>SDG 13 - Climate action</t>
         </is>
@@ -3761,10 +4154,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F61" s="26" t="n"/>
-      <c r="G61" s="26" t="n"/>
-      <c r="H61" s="26" t="n"/>
-      <c r="I61" s="26" t="n">
+      <c r="F61" s="27" t="n"/>
+      <c r="G61" s="27" t="n"/>
+      <c r="H61" s="27" t="n"/>
+      <c r="I61" s="27" t="n">
         <v>15</v>
       </c>
       <c r="J61" s="13" t="inlineStr">
@@ -3785,7 +4178,7 @@
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr"/>
-      <c r="D62" s="25" t="inlineStr">
+      <c r="D62" s="26" t="inlineStr">
         <is>
           <t>SDG 14 - Life below water</t>
         </is>
@@ -3795,10 +4188,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F62" s="26" t="n"/>
-      <c r="G62" s="26" t="n"/>
-      <c r="H62" s="26" t="n"/>
-      <c r="I62" s="26" t="n">
+      <c r="F62" s="27" t="n"/>
+      <c r="G62" s="27" t="n"/>
+      <c r="H62" s="27" t="n"/>
+      <c r="I62" s="27" t="n">
         <v>3</v>
       </c>
       <c r="J62" s="13" t="inlineStr">
@@ -3819,7 +4212,7 @@
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr"/>
-      <c r="D63" s="25" t="inlineStr">
+      <c r="D63" s="26" t="inlineStr">
         <is>
           <t>SDG 15 - Life on land</t>
         </is>
@@ -3829,10 +4222,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F63" s="26" t="n"/>
-      <c r="G63" s="26" t="n"/>
-      <c r="H63" s="26" t="n"/>
-      <c r="I63" s="26" t="n">
+      <c r="F63" s="27" t="n"/>
+      <c r="G63" s="27" t="n"/>
+      <c r="H63" s="27" t="n"/>
+      <c r="I63" s="27" t="n">
         <v>5</v>
       </c>
       <c r="J63" s="13" t="inlineStr">
@@ -3853,7 +4246,7 @@
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr"/>
-      <c r="D64" s="25" t="inlineStr">
+      <c r="D64" s="26" t="inlineStr">
         <is>
           <t>SDG 16 - Peace, justice and strong institutions</t>
         </is>
@@ -3863,10 +4256,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F64" s="26" t="n"/>
-      <c r="G64" s="26" t="n"/>
-      <c r="H64" s="26" t="n"/>
-      <c r="I64" s="26" t="n">
+      <c r="F64" s="27" t="n"/>
+      <c r="G64" s="27" t="n"/>
+      <c r="H64" s="27" t="n"/>
+      <c r="I64" s="27" t="n">
         <v>0</v>
       </c>
       <c r="J64" s="13" t="inlineStr">
@@ -3887,7 +4280,7 @@
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr"/>
-      <c r="D65" s="25" t="inlineStr">
+      <c r="D65" s="26" t="inlineStr">
         <is>
           <t>SDG 17 - Partnerships</t>
         </is>
@@ -3897,10 +4290,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F65" s="26" t="n"/>
-      <c r="G65" s="26" t="n"/>
-      <c r="H65" s="26" t="n"/>
-      <c r="I65" s="26" t="n">
+      <c r="F65" s="27" t="n"/>
+      <c r="G65" s="27" t="n"/>
+      <c r="H65" s="27" t="n"/>
+      <c r="I65" s="27" t="n">
         <v>0</v>
       </c>
       <c r="J65" s="13" t="inlineStr">
@@ -3931,10 +4324,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F66" s="26" t="n"/>
-      <c r="G66" s="26" t="n"/>
-      <c r="H66" s="26" t="n"/>
-      <c r="I66" s="26" t="n">
+      <c r="F66" s="27" t="n"/>
+      <c r="G66" s="27" t="n"/>
+      <c r="H66" s="27" t="n"/>
+      <c r="I66" s="27" t="n">
         <v>1256</v>
       </c>
       <c r="J66" s="13" t="inlineStr">
@@ -3955,7 +4348,7 @@
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr"/>
-      <c r="D67" s="25" t="inlineStr">
+      <c r="D67" s="26" t="inlineStr">
         <is>
           <t>SDG 1 - No Poverty</t>
         </is>
@@ -3965,10 +4358,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F67" s="26" t="n"/>
-      <c r="G67" s="26" t="n"/>
-      <c r="H67" s="26" t="n"/>
-      <c r="I67" s="26" t="n">
+      <c r="F67" s="27" t="n"/>
+      <c r="G67" s="27" t="n"/>
+      <c r="H67" s="27" t="n"/>
+      <c r="I67" s="27" t="n">
         <v>6</v>
       </c>
       <c r="J67" s="13" t="inlineStr">
@@ -3989,7 +4382,7 @@
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr"/>
-      <c r="D68" s="25" t="inlineStr">
+      <c r="D68" s="26" t="inlineStr">
         <is>
           <t>SDG 2 - Zero Hunger</t>
         </is>
@@ -3999,10 +4392,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F68" s="26" t="n"/>
-      <c r="G68" s="26" t="n"/>
-      <c r="H68" s="26" t="n"/>
-      <c r="I68" s="26" t="n">
+      <c r="F68" s="27" t="n"/>
+      <c r="G68" s="27" t="n"/>
+      <c r="H68" s="27" t="n"/>
+      <c r="I68" s="27" t="n">
         <v>32</v>
       </c>
       <c r="J68" s="13" t="inlineStr">
@@ -4023,7 +4416,7 @@
         </is>
       </c>
       <c r="C69" s="13" t="inlineStr"/>
-      <c r="D69" s="25" t="inlineStr">
+      <c r="D69" s="26" t="inlineStr">
         <is>
           <t>SDG 3 - Good health and well-being</t>
         </is>
@@ -4033,10 +4426,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F69" s="26" t="n"/>
-      <c r="G69" s="26" t="n"/>
-      <c r="H69" s="26" t="n"/>
-      <c r="I69" s="26" t="n">
+      <c r="F69" s="27" t="n"/>
+      <c r="G69" s="27" t="n"/>
+      <c r="H69" s="27" t="n"/>
+      <c r="I69" s="27" t="n">
         <v>676</v>
       </c>
       <c r="J69" s="13" t="inlineStr">
@@ -4057,7 +4450,7 @@
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr"/>
-      <c r="D70" s="25" t="inlineStr">
+      <c r="D70" s="26" t="inlineStr">
         <is>
           <t>SDG 4 - Quality Education</t>
         </is>
@@ -4067,10 +4460,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F70" s="26" t="n"/>
-      <c r="G70" s="26" t="n"/>
-      <c r="H70" s="26" t="n"/>
-      <c r="I70" s="26" t="n">
+      <c r="F70" s="27" t="n"/>
+      <c r="G70" s="27" t="n"/>
+      <c r="H70" s="27" t="n"/>
+      <c r="I70" s="27" t="n">
         <v>48</v>
       </c>
       <c r="J70" s="13" t="inlineStr">
@@ -4091,7 +4484,7 @@
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr"/>
-      <c r="D71" s="25" t="inlineStr">
+      <c r="D71" s="26" t="inlineStr">
         <is>
           <t>SDG 5 - Gender Equality</t>
         </is>
@@ -4101,10 +4494,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F71" s="26" t="n"/>
-      <c r="G71" s="26" t="n"/>
-      <c r="H71" s="26" t="n"/>
-      <c r="I71" s="26" t="n">
+      <c r="F71" s="27" t="n"/>
+      <c r="G71" s="27" t="n"/>
+      <c r="H71" s="27" t="n"/>
+      <c r="I71" s="27" t="n">
         <v>30</v>
       </c>
       <c r="J71" s="13" t="inlineStr">
@@ -4125,7 +4518,7 @@
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr"/>
-      <c r="D72" s="25" t="inlineStr">
+      <c r="D72" s="26" t="inlineStr">
         <is>
           <t>SDG 6 - Clean water and sanitation</t>
         </is>
@@ -4135,10 +4528,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F72" s="26" t="n"/>
-      <c r="G72" s="26" t="n"/>
-      <c r="H72" s="26" t="n"/>
-      <c r="I72" s="26" t="n">
+      <c r="F72" s="27" t="n"/>
+      <c r="G72" s="27" t="n"/>
+      <c r="H72" s="27" t="n"/>
+      <c r="I72" s="27" t="n">
         <v>32</v>
       </c>
       <c r="J72" s="13" t="inlineStr">
@@ -4159,7 +4552,7 @@
         </is>
       </c>
       <c r="C73" s="13" t="inlineStr"/>
-      <c r="D73" s="25" t="inlineStr">
+      <c r="D73" s="26" t="inlineStr">
         <is>
           <t>SDG 7 - Affordable and clean energy</t>
         </is>
@@ -4169,10 +4562,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F73" s="26" t="n"/>
-      <c r="G73" s="26" t="n"/>
-      <c r="H73" s="26" t="n"/>
-      <c r="I73" s="26" t="n">
+      <c r="F73" s="27" t="n"/>
+      <c r="G73" s="27" t="n"/>
+      <c r="H73" s="27" t="n"/>
+      <c r="I73" s="27" t="n">
         <v>12</v>
       </c>
       <c r="J73" s="13" t="inlineStr">
@@ -4193,7 +4586,7 @@
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr"/>
-      <c r="D74" s="25" t="inlineStr">
+      <c r="D74" s="26" t="inlineStr">
         <is>
           <t>SDG 8 - Decent work and economic growth</t>
         </is>
@@ -4203,10 +4596,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F74" s="26" t="n"/>
-      <c r="G74" s="26" t="n"/>
-      <c r="H74" s="26" t="n"/>
-      <c r="I74" s="26" t="n">
+      <c r="F74" s="27" t="n"/>
+      <c r="G74" s="27" t="n"/>
+      <c r="H74" s="27" t="n"/>
+      <c r="I74" s="27" t="n">
         <v>31</v>
       </c>
       <c r="J74" s="13" t="inlineStr">
@@ -4227,7 +4620,7 @@
         </is>
       </c>
       <c r="C75" s="13" t="inlineStr"/>
-      <c r="D75" s="25" t="inlineStr">
+      <c r="D75" s="26" t="inlineStr">
         <is>
           <t>SDG 9 - Industry, innovation and infrastructure</t>
         </is>
@@ -4237,10 +4630,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F75" s="26" t="n"/>
-      <c r="G75" s="26" t="n"/>
-      <c r="H75" s="26" t="n"/>
-      <c r="I75" s="26" t="n">
+      <c r="F75" s="27" t="n"/>
+      <c r="G75" s="27" t="n"/>
+      <c r="H75" s="27" t="n"/>
+      <c r="I75" s="27" t="n">
         <v>1</v>
       </c>
       <c r="J75" s="13" t="inlineStr">
@@ -4261,7 +4654,7 @@
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr"/>
-      <c r="D76" s="25" t="inlineStr">
+      <c r="D76" s="26" t="inlineStr">
         <is>
           <t>SDG 10 - Reduced inequality</t>
         </is>
@@ -4271,10 +4664,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F76" s="26" t="n"/>
-      <c r="G76" s="26" t="n"/>
-      <c r="H76" s="26" t="n"/>
-      <c r="I76" s="26" t="n">
+      <c r="F76" s="27" t="n"/>
+      <c r="G76" s="27" t="n"/>
+      <c r="H76" s="27" t="n"/>
+      <c r="I76" s="27" t="n">
         <v>29</v>
       </c>
       <c r="J76" s="13" t="inlineStr">
@@ -4295,7 +4688,7 @@
         </is>
       </c>
       <c r="C77" s="13" t="inlineStr"/>
-      <c r="D77" s="25" t="inlineStr">
+      <c r="D77" s="26" t="inlineStr">
         <is>
           <t>SDG 11 - Sustainable cities and communities</t>
         </is>
@@ -4305,10 +4698,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F77" s="26" t="n"/>
-      <c r="G77" s="26" t="n"/>
-      <c r="H77" s="26" t="n"/>
-      <c r="I77" s="26" t="n">
+      <c r="F77" s="27" t="n"/>
+      <c r="G77" s="27" t="n"/>
+      <c r="H77" s="27" t="n"/>
+      <c r="I77" s="27" t="n">
         <v>27</v>
       </c>
       <c r="J77" s="13" t="inlineStr">
@@ -4329,7 +4722,7 @@
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr"/>
-      <c r="D78" s="25" t="inlineStr">
+      <c r="D78" s="26" t="inlineStr">
         <is>
           <t>SDG 12 - Responsible consumption and production</t>
         </is>
@@ -4339,10 +4732,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F78" s="26" t="n"/>
-      <c r="G78" s="26" t="n"/>
-      <c r="H78" s="26" t="n"/>
-      <c r="I78" s="26" t="n">
+      <c r="F78" s="27" t="n"/>
+      <c r="G78" s="27" t="n"/>
+      <c r="H78" s="27" t="n"/>
+      <c r="I78" s="27" t="n">
         <v>8</v>
       </c>
       <c r="J78" s="13" t="inlineStr">
@@ -4363,7 +4756,7 @@
         </is>
       </c>
       <c r="C79" s="13" t="inlineStr"/>
-      <c r="D79" s="25" t="inlineStr">
+      <c r="D79" s="26" t="inlineStr">
         <is>
           <t>SDG 13 - Climate action</t>
         </is>
@@ -4373,10 +4766,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F79" s="26" t="n"/>
-      <c r="G79" s="26" t="n"/>
-      <c r="H79" s="26" t="n"/>
-      <c r="I79" s="26" t="n">
+      <c r="F79" s="27" t="n"/>
+      <c r="G79" s="27" t="n"/>
+      <c r="H79" s="27" t="n"/>
+      <c r="I79" s="27" t="n">
         <v>193</v>
       </c>
       <c r="J79" s="13" t="inlineStr">
@@ -4397,7 +4790,7 @@
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr"/>
-      <c r="D80" s="25" t="inlineStr">
+      <c r="D80" s="26" t="inlineStr">
         <is>
           <t>SDG 14 - Life below water</t>
         </is>
@@ -4407,10 +4800,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F80" s="26" t="n"/>
-      <c r="G80" s="26" t="n"/>
-      <c r="H80" s="26" t="n"/>
-      <c r="I80" s="26" t="n">
+      <c r="F80" s="27" t="n"/>
+      <c r="G80" s="27" t="n"/>
+      <c r="H80" s="27" t="n"/>
+      <c r="I80" s="27" t="n">
         <v>13</v>
       </c>
       <c r="J80" s="13" t="inlineStr">
@@ -4431,7 +4824,7 @@
         </is>
       </c>
       <c r="C81" s="13" t="inlineStr"/>
-      <c r="D81" s="25" t="inlineStr">
+      <c r="D81" s="26" t="inlineStr">
         <is>
           <t>SDG 15 - Life on land</t>
         </is>
@@ -4441,10 +4834,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F81" s="26" t="n"/>
-      <c r="G81" s="26" t="n"/>
-      <c r="H81" s="26" t="n"/>
-      <c r="I81" s="26" t="n">
+      <c r="F81" s="27" t="n"/>
+      <c r="G81" s="27" t="n"/>
+      <c r="H81" s="27" t="n"/>
+      <c r="I81" s="27" t="n">
         <v>65</v>
       </c>
       <c r="J81" s="13" t="inlineStr">
@@ -4465,7 +4858,7 @@
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr"/>
-      <c r="D82" s="25" t="inlineStr">
+      <c r="D82" s="26" t="inlineStr">
         <is>
           <t>SDG 16 - Peace, justice and strong institutions</t>
         </is>
@@ -4475,10 +4868,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F82" s="26" t="n"/>
-      <c r="G82" s="26" t="n"/>
-      <c r="H82" s="26" t="n"/>
-      <c r="I82" s="26" t="n">
+      <c r="F82" s="27" t="n"/>
+      <c r="G82" s="27" t="n"/>
+      <c r="H82" s="27" t="n"/>
+      <c r="I82" s="27" t="n">
         <v>52</v>
       </c>
       <c r="J82" s="13" t="inlineStr">
@@ -4499,7 +4892,7 @@
         </is>
       </c>
       <c r="C83" s="13" t="inlineStr"/>
-      <c r="D83" s="25" t="inlineStr">
+      <c r="D83" s="26" t="inlineStr">
         <is>
           <t>SDG 17 - Partnerships</t>
         </is>
@@ -4509,10 +4902,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F83" s="26" t="n"/>
-      <c r="G83" s="26" t="n"/>
-      <c r="H83" s="26" t="n"/>
-      <c r="I83" s="26" t="n">
+      <c r="F83" s="27" t="n"/>
+      <c r="G83" s="27" t="n"/>
+      <c r="H83" s="27" t="n"/>
+      <c r="I83" s="27" t="n">
         <v>1</v>
       </c>
       <c r="J83" s="13" t="inlineStr">
@@ -4543,10 +4936,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F84" s="26" t="n"/>
-      <c r="G84" s="26" t="n"/>
-      <c r="H84" s="26" t="n"/>
-      <c r="I84" s="26" t="n">
+      <c r="F84" s="27" t="n"/>
+      <c r="G84" s="27" t="n"/>
+      <c r="H84" s="27" t="n"/>
+      <c r="I84" s="27" t="n">
         <v>86993</v>
       </c>
       <c r="J84" s="13" t="inlineStr">
@@ -4567,7 +4960,7 @@
         </is>
       </c>
       <c r="C85" s="13" t="inlineStr"/>
-      <c r="D85" s="25" t="inlineStr">
+      <c r="D85" s="26" t="inlineStr">
         <is>
           <t>SDG 1 - No Poverty</t>
         </is>
@@ -4577,10 +4970,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F85" s="26" t="n"/>
-      <c r="G85" s="26" t="n"/>
-      <c r="H85" s="26" t="n"/>
-      <c r="I85" s="26" t="n">
+      <c r="F85" s="27" t="n"/>
+      <c r="G85" s="27" t="n"/>
+      <c r="H85" s="27" t="n"/>
+      <c r="I85" s="27" t="n">
         <v>17</v>
       </c>
       <c r="J85" s="13" t="inlineStr">
@@ -4601,7 +4994,7 @@
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr"/>
-      <c r="D86" s="25" t="inlineStr">
+      <c r="D86" s="26" t="inlineStr">
         <is>
           <t>SDG 2 - Zero Hunger</t>
         </is>
@@ -4611,10 +5004,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F86" s="26" t="n"/>
-      <c r="G86" s="26" t="n"/>
-      <c r="H86" s="26" t="n"/>
-      <c r="I86" s="26" t="n">
+      <c r="F86" s="27" t="n"/>
+      <c r="G86" s="27" t="n"/>
+      <c r="H86" s="27" t="n"/>
+      <c r="I86" s="27" t="n">
         <v>731</v>
       </c>
       <c r="J86" s="13" t="inlineStr">
@@ -4635,7 +5028,7 @@
         </is>
       </c>
       <c r="C87" s="13" t="inlineStr"/>
-      <c r="D87" s="25" t="inlineStr">
+      <c r="D87" s="26" t="inlineStr">
         <is>
           <t>SDG 3 - Good health and well-being</t>
         </is>
@@ -4645,10 +5038,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F87" s="26" t="n"/>
-      <c r="G87" s="26" t="n"/>
-      <c r="H87" s="26" t="n"/>
-      <c r="I87" s="26" t="n">
+      <c r="F87" s="27" t="n"/>
+      <c r="G87" s="27" t="n"/>
+      <c r="H87" s="27" t="n"/>
+      <c r="I87" s="27" t="n">
         <v>55989</v>
       </c>
       <c r="J87" s="13" t="inlineStr">
@@ -4669,7 +5062,7 @@
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr"/>
-      <c r="D88" s="25" t="inlineStr">
+      <c r="D88" s="26" t="inlineStr">
         <is>
           <t>SDG 4 - Quality Education</t>
         </is>
@@ -4679,10 +5072,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F88" s="26" t="n"/>
-      <c r="G88" s="26" t="n"/>
-      <c r="H88" s="26" t="n"/>
-      <c r="I88" s="26" t="n">
+      <c r="F88" s="27" t="n"/>
+      <c r="G88" s="27" t="n"/>
+      <c r="H88" s="27" t="n"/>
+      <c r="I88" s="27" t="n">
         <v>6263</v>
       </c>
       <c r="J88" s="13" t="inlineStr">
@@ -4703,7 +5096,7 @@
         </is>
       </c>
       <c r="C89" s="13" t="inlineStr"/>
-      <c r="D89" s="25" t="inlineStr">
+      <c r="D89" s="26" t="inlineStr">
         <is>
           <t>SDG 5 - Gender Equality</t>
         </is>
@@ -4713,10 +5106,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F89" s="26" t="n"/>
-      <c r="G89" s="26" t="n"/>
-      <c r="H89" s="26" t="n"/>
-      <c r="I89" s="26" t="n">
+      <c r="F89" s="27" t="n"/>
+      <c r="G89" s="27" t="n"/>
+      <c r="H89" s="27" t="n"/>
+      <c r="I89" s="27" t="n">
         <v>5286</v>
       </c>
       <c r="J89" s="13" t="inlineStr">
@@ -4737,7 +5130,7 @@
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr"/>
-      <c r="D90" s="25" t="inlineStr">
+      <c r="D90" s="26" t="inlineStr">
         <is>
           <t>SDG 6 - Clean water and sanitation</t>
         </is>
@@ -4747,10 +5140,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F90" s="26" t="n"/>
-      <c r="G90" s="26" t="n"/>
-      <c r="H90" s="26" t="n"/>
-      <c r="I90" s="26" t="n">
+      <c r="F90" s="27" t="n"/>
+      <c r="G90" s="27" t="n"/>
+      <c r="H90" s="27" t="n"/>
+      <c r="I90" s="27" t="n">
         <v>248</v>
       </c>
       <c r="J90" s="13" t="inlineStr">
@@ -4771,7 +5164,7 @@
         </is>
       </c>
       <c r="C91" s="13" t="inlineStr"/>
-      <c r="D91" s="25" t="inlineStr">
+      <c r="D91" s="26" t="inlineStr">
         <is>
           <t>SDG 7 - Affordable and clean energy</t>
         </is>
@@ -4781,10 +5174,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F91" s="26" t="n"/>
-      <c r="G91" s="26" t="n"/>
-      <c r="H91" s="26" t="n"/>
-      <c r="I91" s="26" t="n">
+      <c r="F91" s="27" t="n"/>
+      <c r="G91" s="27" t="n"/>
+      <c r="H91" s="27" t="n"/>
+      <c r="I91" s="27" t="n">
         <v>1009</v>
       </c>
       <c r="J91" s="13" t="inlineStr">
@@ -4805,7 +5198,7 @@
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr"/>
-      <c r="D92" s="25" t="inlineStr">
+      <c r="D92" s="26" t="inlineStr">
         <is>
           <t>SDG 8 - Decent work and economic growth</t>
         </is>
@@ -4815,10 +5208,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F92" s="26" t="n"/>
-      <c r="G92" s="26" t="n"/>
-      <c r="H92" s="26" t="n"/>
-      <c r="I92" s="26" t="n">
+      <c r="F92" s="27" t="n"/>
+      <c r="G92" s="27" t="n"/>
+      <c r="H92" s="27" t="n"/>
+      <c r="I92" s="27" t="n">
         <v>844</v>
       </c>
       <c r="J92" s="13" t="inlineStr">
@@ -4839,7 +5232,7 @@
         </is>
       </c>
       <c r="C93" s="13" t="inlineStr"/>
-      <c r="D93" s="25" t="inlineStr">
+      <c r="D93" s="26" t="inlineStr">
         <is>
           <t>SDG 9 - Industry, innovation and infrastructure</t>
         </is>
@@ -4849,10 +5242,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F93" s="26" t="n"/>
-      <c r="G93" s="26" t="n"/>
-      <c r="H93" s="26" t="n"/>
-      <c r="I93" s="26" t="n">
+      <c r="F93" s="27" t="n"/>
+      <c r="G93" s="27" t="n"/>
+      <c r="H93" s="27" t="n"/>
+      <c r="I93" s="27" t="n">
         <v>48</v>
       </c>
       <c r="J93" s="13" t="inlineStr">
@@ -4873,7 +5266,7 @@
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr"/>
-      <c r="D94" s="25" t="inlineStr">
+      <c r="D94" s="26" t="inlineStr">
         <is>
           <t>SDG 10 - Reduced inequality</t>
         </is>
@@ -4883,10 +5276,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F94" s="26" t="n"/>
-      <c r="G94" s="26" t="n"/>
-      <c r="H94" s="26" t="n"/>
-      <c r="I94" s="26" t="n">
+      <c r="F94" s="27" t="n"/>
+      <c r="G94" s="27" t="n"/>
+      <c r="H94" s="27" t="n"/>
+      <c r="I94" s="27" t="n">
         <v>1032</v>
       </c>
       <c r="J94" s="13" t="inlineStr">
@@ -4907,7 +5300,7 @@
         </is>
       </c>
       <c r="C95" s="13" t="inlineStr"/>
-      <c r="D95" s="25" t="inlineStr">
+      <c r="D95" s="26" t="inlineStr">
         <is>
           <t>SDG 11 - Sustainable cities and communities</t>
         </is>
@@ -4917,10 +5310,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F95" s="26" t="n"/>
-      <c r="G95" s="26" t="n"/>
-      <c r="H95" s="26" t="n"/>
-      <c r="I95" s="26" t="n">
+      <c r="F95" s="27" t="n"/>
+      <c r="G95" s="27" t="n"/>
+      <c r="H95" s="27" t="n"/>
+      <c r="I95" s="27" t="n">
         <v>400</v>
       </c>
       <c r="J95" s="13" t="inlineStr">
@@ -4941,7 +5334,7 @@
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr"/>
-      <c r="D96" s="25" t="inlineStr">
+      <c r="D96" s="26" t="inlineStr">
         <is>
           <t>SDG 12 - Responsible consumption and production</t>
         </is>
@@ -4951,10 +5344,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F96" s="26" t="n"/>
-      <c r="G96" s="26" t="n"/>
-      <c r="H96" s="26" t="n"/>
-      <c r="I96" s="26" t="n">
+      <c r="F96" s="27" t="n"/>
+      <c r="G96" s="27" t="n"/>
+      <c r="H96" s="27" t="n"/>
+      <c r="I96" s="27" t="n">
         <v>224</v>
       </c>
       <c r="J96" s="13" t="inlineStr">
@@ -4975,7 +5368,7 @@
         </is>
       </c>
       <c r="C97" s="13" t="inlineStr"/>
-      <c r="D97" s="25" t="inlineStr">
+      <c r="D97" s="26" t="inlineStr">
         <is>
           <t>SDG 13 - Climate action</t>
         </is>
@@ -4985,10 +5378,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F97" s="26" t="n"/>
-      <c r="G97" s="26" t="n"/>
-      <c r="H97" s="26" t="n"/>
-      <c r="I97" s="26" t="n">
+      <c r="F97" s="27" t="n"/>
+      <c r="G97" s="27" t="n"/>
+      <c r="H97" s="27" t="n"/>
+      <c r="I97" s="27" t="n">
         <v>9639</v>
       </c>
       <c r="J97" s="13" t="inlineStr">
@@ -5009,7 +5402,7 @@
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr"/>
-      <c r="D98" s="25" t="inlineStr">
+      <c r="D98" s="26" t="inlineStr">
         <is>
           <t>SDG 14 - Life below water</t>
         </is>
@@ -5019,10 +5412,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F98" s="26" t="n"/>
-      <c r="G98" s="26" t="n"/>
-      <c r="H98" s="26" t="n"/>
-      <c r="I98" s="26" t="n">
+      <c r="F98" s="27" t="n"/>
+      <c r="G98" s="27" t="n"/>
+      <c r="H98" s="27" t="n"/>
+      <c r="I98" s="27" t="n">
         <v>1503</v>
       </c>
       <c r="J98" s="13" t="inlineStr">
@@ -5043,7 +5436,7 @@
         </is>
       </c>
       <c r="C99" s="13" t="inlineStr"/>
-      <c r="D99" s="25" t="inlineStr">
+      <c r="D99" s="26" t="inlineStr">
         <is>
           <t>SDG 15 - Life on land</t>
         </is>
@@ -5053,10 +5446,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F99" s="26" t="n"/>
-      <c r="G99" s="26" t="n"/>
-      <c r="H99" s="26" t="n"/>
-      <c r="I99" s="26" t="n">
+      <c r="F99" s="27" t="n"/>
+      <c r="G99" s="27" t="n"/>
+      <c r="H99" s="27" t="n"/>
+      <c r="I99" s="27" t="n">
         <v>2844</v>
       </c>
       <c r="J99" s="13" t="inlineStr">
@@ -5077,7 +5470,7 @@
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr"/>
-      <c r="D100" s="25" t="inlineStr">
+      <c r="D100" s="26" t="inlineStr">
         <is>
           <t>SDG 16 - Peace, justice and strong institutions</t>
         </is>
@@ -5087,10 +5480,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F100" s="26" t="n"/>
-      <c r="G100" s="26" t="n"/>
-      <c r="H100" s="26" t="n"/>
-      <c r="I100" s="26" t="n">
+      <c r="F100" s="27" t="n"/>
+      <c r="G100" s="27" t="n"/>
+      <c r="H100" s="27" t="n"/>
+      <c r="I100" s="27" t="n">
         <v>916</v>
       </c>
       <c r="J100" s="13" t="inlineStr">
@@ -5111,7 +5504,7 @@
         </is>
       </c>
       <c r="C101" s="13" t="inlineStr"/>
-      <c r="D101" s="25" t="inlineStr">
+      <c r="D101" s="26" t="inlineStr">
         <is>
           <t>SDG 17 - Partnerships</t>
         </is>
@@ -5121,10 +5514,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F101" s="26" t="n"/>
-      <c r="G101" s="26" t="n"/>
-      <c r="H101" s="26" t="n"/>
-      <c r="I101" s="26" t="n">
+      <c r="F101" s="27" t="n"/>
+      <c r="G101" s="27" t="n"/>
+      <c r="H101" s="27" t="n"/>
+      <c r="I101" s="27" t="n">
         <v>0</v>
       </c>
       <c r="J101" s="13" t="inlineStr">
@@ -5159,20 +5552,20 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F102" s="26" t="n"/>
-      <c r="G102" s="26" t="n"/>
-      <c r="H102" s="26" t="n"/>
-      <c r="I102" s="26" t="n"/>
+      <c r="F102" s="27" t="n"/>
+      <c r="G102" s="27" t="n"/>
+      <c r="H102" s="27" t="n"/>
+      <c r="I102" s="27" t="n"/>
       <c r="J102" s="13" t="inlineStr">
         <is>
           <t>New – no data yet</t>
         </is>
       </c>
-      <c r="K102" s="14" t="n"/>
-      <c r="L102" s="14" t="n"/>
-      <c r="M102" s="14" t="n"/>
-      <c r="N102" s="14" t="n"/>
-      <c r="O102" s="14" t="n"/>
+      <c r="K102" s="15" t="n"/>
+      <c r="L102" s="15" t="n"/>
+      <c r="M102" s="15" t="n"/>
+      <c r="N102" s="15" t="n"/>
+      <c r="O102" s="15" t="n"/>
     </row>
     <row r="103" ht="39" customHeight="1">
       <c r="B103" s="11" t="inlineStr">
@@ -5191,10 +5584,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F103" s="26" t="n"/>
-      <c r="G103" s="26" t="n"/>
-      <c r="H103" s="26" t="n"/>
-      <c r="I103" s="26" t="n"/>
+      <c r="F103" s="27" t="n"/>
+      <c r="G103" s="27" t="n"/>
+      <c r="H103" s="27" t="n"/>
+      <c r="I103" s="27" t="n"/>
       <c r="J103" s="13" t="inlineStr">
         <is>
           <t>New – no data yet</t>
@@ -5223,10 +5616,10 @@
           <t>#</t>
         </is>
       </c>
-      <c r="F104" s="26" t="n"/>
-      <c r="G104" s="26" t="n"/>
-      <c r="H104" s="26" t="n"/>
-      <c r="I104" s="26" t="n"/>
+      <c r="F104" s="27" t="n"/>
+      <c r="G104" s="27" t="n"/>
+      <c r="H104" s="27" t="n"/>
+      <c r="I104" s="27" t="n"/>
       <c r="J104" s="13" t="inlineStr">
         <is>
           <t>New – no data yet</t>
@@ -5237,234 +5630,6 @@
       <c r="M104" s="13" t="n"/>
       <c r="N104" s="13" t="n"/>
       <c r="O104" s="13" t="n"/>
-    </row>
-    <row r="105" ht="39" customHeight="1">
-      <c r="B105" s="11" t="inlineStr">
-        <is>
-          <t>NB2(a)</t>
-        </is>
-      </c>
-      <c r="C105" s="13" t="inlineStr">
-        <is>
-          <t>Documented baseline nature footprint analysis</t>
-        </is>
-      </c>
-      <c r="D105" s="13" t="inlineStr">
-        <is>
-          <t>Freshwater eutrophication</t>
-        </is>
-      </c>
-      <c r="E105" s="13" t="inlineStr">
-        <is>
-          <t>kg P eq</t>
-        </is>
-      </c>
-      <c r="F105" s="26" t="n"/>
-      <c r="G105" s="26" t="n"/>
-      <c r="H105" s="26" t="n"/>
-      <c r="I105" s="26" t="n"/>
-      <c r="J105" s="13" t="inlineStr">
-        <is>
-          <t>New – no data yet</t>
-        </is>
-      </c>
-      <c r="K105" s="14" t="n"/>
-      <c r="L105" s="14" t="n"/>
-      <c r="M105" s="14" t="n"/>
-      <c r="N105" s="14" t="n"/>
-      <c r="O105" s="14" t="n"/>
-    </row>
-    <row r="106" ht="39" customHeight="1">
-      <c r="B106" s="11" t="inlineStr">
-        <is>
-          <t>NB2(a)</t>
-        </is>
-      </c>
-      <c r="C106" s="13" t="inlineStr"/>
-      <c r="D106" s="13" t="inlineStr">
-        <is>
-          <t>Global warming</t>
-        </is>
-      </c>
-      <c r="E106" s="13" t="inlineStr">
-        <is>
-          <t>kg CO2 eq</t>
-        </is>
-      </c>
-      <c r="F106" s="26" t="n"/>
-      <c r="G106" s="26" t="n"/>
-      <c r="H106" s="26" t="n"/>
-      <c r="I106" s="26" t="n"/>
-      <c r="J106" s="13" t="inlineStr">
-        <is>
-          <t>New – no data yet</t>
-        </is>
-      </c>
-      <c r="K106" s="13" t="n"/>
-      <c r="L106" s="13" t="n"/>
-      <c r="M106" s="13" t="n"/>
-      <c r="N106" s="13" t="n"/>
-      <c r="O106" s="13" t="n"/>
-    </row>
-    <row r="107" ht="39" customHeight="1">
-      <c r="B107" s="11" t="inlineStr">
-        <is>
-          <t>NB2(a)</t>
-        </is>
-      </c>
-      <c r="C107" s="13" t="inlineStr"/>
-      <c r="D107" s="13" t="inlineStr">
-        <is>
-          <t>Land use</t>
-        </is>
-      </c>
-      <c r="E107" s="13" t="inlineStr">
-        <is>
-          <t>m²a crop eq</t>
-        </is>
-      </c>
-      <c r="F107" s="26" t="n"/>
-      <c r="G107" s="26" t="n"/>
-      <c r="H107" s="26" t="n"/>
-      <c r="I107" s="26" t="n"/>
-      <c r="J107" s="13" t="inlineStr">
-        <is>
-          <t>New – no data yet</t>
-        </is>
-      </c>
-      <c r="K107" s="13" t="n"/>
-      <c r="L107" s="13" t="n"/>
-      <c r="M107" s="13" t="n"/>
-      <c r="N107" s="13" t="n"/>
-      <c r="O107" s="13" t="n"/>
-    </row>
-    <row r="108" ht="39" customHeight="1">
-      <c r="B108" s="11" t="inlineStr">
-        <is>
-          <t>NB2(a)</t>
-        </is>
-      </c>
-      <c r="C108" s="13" t="inlineStr"/>
-      <c r="D108" s="13" t="inlineStr">
-        <is>
-          <t>Marine eutrophication</t>
-        </is>
-      </c>
-      <c r="E108" s="13" t="inlineStr">
-        <is>
-          <t>kg N eq</t>
-        </is>
-      </c>
-      <c r="F108" s="26" t="n"/>
-      <c r="G108" s="26" t="n"/>
-      <c r="H108" s="26" t="n"/>
-      <c r="I108" s="26" t="n"/>
-      <c r="J108" s="13" t="inlineStr">
-        <is>
-          <t>New – no data yet</t>
-        </is>
-      </c>
-      <c r="K108" s="13" t="n"/>
-      <c r="L108" s="13" t="n"/>
-      <c r="M108" s="13" t="n"/>
-      <c r="N108" s="13" t="n"/>
-      <c r="O108" s="13" t="n"/>
-    </row>
-    <row r="109" ht="39" customHeight="1">
-      <c r="B109" s="11" t="inlineStr">
-        <is>
-          <t>NB2(a)</t>
-        </is>
-      </c>
-      <c r="C109" s="13" t="inlineStr"/>
-      <c r="D109" s="13" t="inlineStr">
-        <is>
-          <t>Photochemical ozone formation</t>
-        </is>
-      </c>
-      <c r="E109" s="13" t="inlineStr">
-        <is>
-          <t>kg NOx eq</t>
-        </is>
-      </c>
-      <c r="F109" s="26" t="n"/>
-      <c r="G109" s="26" t="n"/>
-      <c r="H109" s="26" t="n"/>
-      <c r="I109" s="26" t="n"/>
-      <c r="J109" s="13" t="inlineStr">
-        <is>
-          <t>New – no data yet</t>
-        </is>
-      </c>
-      <c r="K109" s="13" t="n"/>
-      <c r="L109" s="13" t="n"/>
-      <c r="M109" s="13" t="n"/>
-      <c r="N109" s="13" t="n"/>
-      <c r="O109" s="13" t="n"/>
-    </row>
-    <row r="110" ht="39" customHeight="1">
-      <c r="B110" s="11" t="inlineStr">
-        <is>
-          <t>NB2(a)</t>
-        </is>
-      </c>
-      <c r="C110" s="13" t="inlineStr"/>
-      <c r="D110" s="13" t="inlineStr">
-        <is>
-          <t>Terrestrial acidification</t>
-        </is>
-      </c>
-      <c r="E110" s="13" t="inlineStr">
-        <is>
-          <t>kg SO2 eq</t>
-        </is>
-      </c>
-      <c r="F110" s="26" t="n"/>
-      <c r="G110" s="26" t="n"/>
-      <c r="H110" s="26" t="n"/>
-      <c r="I110" s="26" t="n"/>
-      <c r="J110" s="13" t="inlineStr">
-        <is>
-          <t>New – no data yet</t>
-        </is>
-      </c>
-      <c r="K110" s="13" t="n"/>
-      <c r="L110" s="13" t="n"/>
-      <c r="M110" s="13" t="n"/>
-      <c r="N110" s="13" t="n"/>
-      <c r="O110" s="13" t="n"/>
-    </row>
-    <row r="111" ht="39" customHeight="1">
-      <c r="B111" s="11" t="inlineStr">
-        <is>
-          <t>NB2(a)</t>
-        </is>
-      </c>
-      <c r="C111" s="13" t="inlineStr"/>
-      <c r="D111" s="13" t="inlineStr">
-        <is>
-          <t>Water consumption</t>
-        </is>
-      </c>
-      <c r="E111" s="13" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="F111" s="26" t="n"/>
-      <c r="G111" s="26" t="n"/>
-      <c r="H111" s="26" t="n"/>
-      <c r="I111" s="26" t="n"/>
-      <c r="J111" s="13" t="inlineStr">
-        <is>
-          <t>New – no data yet</t>
-        </is>
-      </c>
-      <c r="K111" s="13" t="n"/>
-      <c r="L111" s="13" t="n"/>
-      <c r="M111" s="13" t="n"/>
-      <c r="N111" s="13" t="n"/>
-      <c r="O111" s="13" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
@@ -5474,7 +5639,7 @@
     <mergeCell ref="K5:O5"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="M8:M112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Please select from the dropdown" type="list">
+    <dataValidation sqref="M8:M105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Please select from the dropdown" type="list">
       <formula1>"No change,Yes – see notes"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>